<commit_message>
added tender starts; updated prod cap; fixing bad constraint
</commit_message>
<xml_diff>
--- a/production_capacity_updated.xlsx
+++ b/production_capacity_updated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27126"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fthcn\Desktop\Vaccine_Tender_Scheduling_Problem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{391AB4AD-8E06-448B-8305-29E04006C88F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{391AB4AD-8E06-448B-8305-29E04006C88F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{318C915B-7EBB-4C2E-AB54-76CE7BB3ECDA}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="4" xr2:uid="{752E71BE-3FD4-4CCA-ABF0-6C5710D300B4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="4" xr2:uid="{752E71BE-3FD4-4CCA-ABF0-6C5710D300B4}"/>
   </bookViews>
   <sheets>
     <sheet name="vaccine-producer list" sheetId="8" r:id="rId1"/>
@@ -27,9 +27,9 @@
     <definedName name="GAVI_countries" localSheetId="0">#REF!</definedName>
     <definedName name="GAVI_countries">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="191029" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId6"/>
+    <pivotCache cacheId="4" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1798,7 +1798,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B95A2301-B56D-4CF8-964C-AEC6E5E61117}" name="PivotTable3" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B95A2301-B56D-4CF8-964C-AEC6E5E61117}" name="PivotTable3" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="M3:W22" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField axis="axisRow" showAll="0">
@@ -1957,9 +1957,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1997,7 +1997,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2103,7 +2103,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2245,7 +2245,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2306,14 +2306,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3694F37-B2B5-4F9D-9ACD-67519624FADB}">
   <dimension ref="A1:T54"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="91.109375" customWidth="1"/>
-    <col min="2" max="18" width="15.6640625" customWidth="1"/>
-    <col min="20" max="20" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="91.140625" customWidth="1"/>
+    <col min="2" max="18" width="15.7109375" customWidth="1"/>
+    <col min="20" max="20" width="11.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" ht="60" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
@@ -2375,7 +2375,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>43</v>
       </c>
@@ -2403,7 +2403,7 @@
       <c r="S2" s="34"/>
       <c r="T2" s="34"/>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
         <v>92</v>
       </c>
@@ -2431,7 +2431,7 @@
       <c r="S3" s="34"/>
       <c r="T3" s="34"/>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
         <v>93</v>
       </c>
@@ -2459,7 +2459,7 @@
       <c r="S4" s="34"/>
       <c r="T4" s="34"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>94</v>
       </c>
@@ -2489,7 +2489,7 @@
       <c r="S5" s="34"/>
       <c r="T5" s="34"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
         <v>95</v>
       </c>
@@ -2519,7 +2519,7 @@
       <c r="S6" s="34"/>
       <c r="T6" s="34"/>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>96</v>
       </c>
@@ -2549,7 +2549,7 @@
       <c r="S7" s="34"/>
       <c r="T7" s="34"/>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
         <v>157</v>
       </c>
@@ -2583,7 +2583,7 @@
       <c r="S8" s="34"/>
       <c r="T8" s="34"/>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
         <v>97</v>
       </c>
@@ -2611,7 +2611,7 @@
       <c r="S9" s="34"/>
       <c r="T9" s="34"/>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>98</v>
       </c>
@@ -2637,7 +2637,7 @@
       <c r="S10" s="34"/>
       <c r="T10" s="34"/>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
         <v>99</v>
       </c>
@@ -2671,7 +2671,7 @@
       <c r="S11" s="34"/>
       <c r="T11" s="34"/>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
         <v>100</v>
       </c>
@@ -2697,7 +2697,7 @@
       <c r="S12" s="34"/>
       <c r="T12" s="34"/>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
         <v>101</v>
       </c>
@@ -2729,7 +2729,7 @@
       <c r="S13" s="34"/>
       <c r="T13" s="34"/>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="11" t="s">
         <v>102</v>
       </c>
@@ -2769,7 +2769,7 @@
       <c r="S14" s="34"/>
       <c r="T14" s="34"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A15" s="11" t="s">
         <v>103</v>
       </c>
@@ -2801,7 +2801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A16" s="11" t="s">
         <v>104</v>
       </c>
@@ -2829,7 +2829,7 @@
       <c r="S16" s="34"/>
       <c r="T16" s="34"/>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
         <v>105</v>
       </c>
@@ -2859,7 +2859,7 @@
       <c r="S17" s="34"/>
       <c r="T17" s="34"/>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
         <v>158</v>
       </c>
@@ -2889,7 +2889,7 @@
       <c r="S18" s="10"/>
       <c r="T18" s="10"/>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A19" s="11" t="s">
         <v>155</v>
       </c>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="T19" s="10"/>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A20" s="14"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
@@ -2939,7 +2939,7 @@
       <c r="Q20" s="13"/>
       <c r="R20" s="13"/>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
       <c r="D21" s="13"/>
@@ -2958,7 +2958,7 @@
       <c r="Q21" s="13"/>
       <c r="R21" s="13"/>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
       <c r="D22" s="13"/>
@@ -2977,7 +2977,7 @@
       <c r="Q22" s="13"/>
       <c r="R22" s="13"/>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
       <c r="D23" s="13"/>
@@ -2996,7 +2996,7 @@
       <c r="Q23" s="13"/>
       <c r="R23" s="13"/>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
@@ -3015,7 +3015,7 @@
       <c r="Q24" s="13"/>
       <c r="R24" s="13"/>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
       <c r="D25" s="13"/>
@@ -3034,7 +3034,7 @@
       <c r="Q25" s="13"/>
       <c r="R25" s="13"/>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
       <c r="D26" s="13"/>
@@ -3053,7 +3053,7 @@
       <c r="Q26" s="13"/>
       <c r="R26" s="13"/>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
       <c r="D27" s="13"/>
@@ -3072,7 +3072,7 @@
       <c r="Q27" s="13"/>
       <c r="R27" s="13"/>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
       <c r="D28" s="13"/>
@@ -3091,7 +3091,7 @@
       <c r="Q28" s="13"/>
       <c r="R28" s="13"/>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
       <c r="D29" s="13"/>
@@ -3110,7 +3110,7 @@
       <c r="Q29" s="13"/>
       <c r="R29" s="13"/>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B30" s="13"/>
       <c r="C30" s="13"/>
       <c r="D30" s="13"/>
@@ -3129,7 +3129,7 @@
       <c r="Q30" s="13"/>
       <c r="R30" s="13"/>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B31" s="13"/>
       <c r="C31" s="13"/>
       <c r="D31" s="13"/>
@@ -3148,7 +3148,7 @@
       <c r="Q31" s="13"/>
       <c r="R31" s="13"/>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
       <c r="B32" s="13"/>
       <c r="C32" s="13"/>
       <c r="D32" s="13"/>
@@ -3167,7 +3167,7 @@
       <c r="Q32" s="13"/>
       <c r="R32" s="13"/>
     </row>
-    <row r="33" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B33" s="13"/>
       <c r="C33" s="13"/>
       <c r="D33" s="13"/>
@@ -3186,7 +3186,7 @@
       <c r="Q33" s="13"/>
       <c r="R33" s="13"/>
     </row>
-    <row r="34" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B34" s="13"/>
       <c r="C34" s="13"/>
       <c r="D34" s="13"/>
@@ -3205,7 +3205,7 @@
       <c r="Q34" s="13"/>
       <c r="R34" s="13"/>
     </row>
-    <row r="35" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B35" s="13"/>
       <c r="C35" s="13"/>
       <c r="D35" s="13"/>
@@ -3224,7 +3224,7 @@
       <c r="Q35" s="13"/>
       <c r="R35" s="13"/>
     </row>
-    <row r="36" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B36" s="13"/>
       <c r="C36" s="13"/>
       <c r="D36" s="13"/>
@@ -3243,7 +3243,7 @@
       <c r="Q36" s="13"/>
       <c r="R36" s="13"/>
     </row>
-    <row r="37" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B37" s="13"/>
       <c r="C37" s="13"/>
       <c r="D37" s="13"/>
@@ -3262,7 +3262,7 @@
       <c r="Q37" s="13"/>
       <c r="R37" s="13"/>
     </row>
-    <row r="38" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B38" s="13"/>
       <c r="C38" s="13"/>
       <c r="D38" s="13"/>
@@ -3281,7 +3281,7 @@
       <c r="Q38" s="13"/>
       <c r="R38" s="13"/>
     </row>
-    <row r="39" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B39" s="13"/>
       <c r="C39" s="13"/>
       <c r="D39" s="13"/>
@@ -3300,7 +3300,7 @@
       <c r="Q39" s="13"/>
       <c r="R39" s="13"/>
     </row>
-    <row r="40" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B40" s="13"/>
       <c r="C40" s="13"/>
       <c r="D40" s="13"/>
@@ -3319,7 +3319,7 @@
       <c r="Q40" s="13"/>
       <c r="R40" s="13"/>
     </row>
-    <row r="41" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B41" s="13"/>
       <c r="C41" s="13"/>
       <c r="D41" s="13"/>
@@ -3338,7 +3338,7 @@
       <c r="Q41" s="13"/>
       <c r="R41" s="13"/>
     </row>
-    <row r="42" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B42" s="13"/>
       <c r="C42" s="13"/>
       <c r="D42" s="13"/>
@@ -3357,7 +3357,7 @@
       <c r="Q42" s="13"/>
       <c r="R42" s="13"/>
     </row>
-    <row r="43" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B43" s="13"/>
       <c r="C43" s="13"/>
       <c r="D43" s="13"/>
@@ -3376,7 +3376,7 @@
       <c r="Q43" s="13"/>
       <c r="R43" s="13"/>
     </row>
-    <row r="44" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B44" s="13"/>
       <c r="C44" s="13"/>
       <c r="D44" s="13"/>
@@ -3395,7 +3395,7 @@
       <c r="Q44" s="13"/>
       <c r="R44" s="13"/>
     </row>
-    <row r="45" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="45" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B45" s="13"/>
       <c r="C45" s="13"/>
       <c r="D45" s="13"/>
@@ -3414,7 +3414,7 @@
       <c r="Q45" s="13"/>
       <c r="R45" s="13"/>
     </row>
-    <row r="46" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B46" s="13"/>
       <c r="C46" s="13"/>
       <c r="D46" s="13"/>
@@ -3433,7 +3433,7 @@
       <c r="Q46" s="13"/>
       <c r="R46" s="13"/>
     </row>
-    <row r="47" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="47" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B47" s="13"/>
       <c r="C47" s="13"/>
       <c r="D47" s="13"/>
@@ -3452,7 +3452,7 @@
       <c r="Q47" s="13"/>
       <c r="R47" s="13"/>
     </row>
-    <row r="48" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="48" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B48" s="13"/>
       <c r="C48" s="13"/>
       <c r="D48" s="13"/>
@@ -3471,7 +3471,7 @@
       <c r="Q48" s="13"/>
       <c r="R48" s="13"/>
     </row>
-    <row r="49" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="49" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B49" s="13"/>
       <c r="C49" s="13"/>
       <c r="D49" s="13"/>
@@ -3490,7 +3490,7 @@
       <c r="Q49" s="13"/>
       <c r="R49" s="13"/>
     </row>
-    <row r="50" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="50" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B50" s="13"/>
       <c r="C50" s="13"/>
       <c r="D50" s="13"/>
@@ -3509,7 +3509,7 @@
       <c r="Q50" s="13"/>
       <c r="R50" s="13"/>
     </row>
-    <row r="51" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B51" s="13"/>
       <c r="C51" s="13"/>
       <c r="D51" s="13"/>
@@ -3528,7 +3528,7 @@
       <c r="Q51" s="13"/>
       <c r="R51" s="13"/>
     </row>
-    <row r="52" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="52" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B52" s="13"/>
       <c r="C52" s="13"/>
       <c r="D52" s="13"/>
@@ -3547,7 +3547,7 @@
       <c r="Q52" s="13"/>
       <c r="R52" s="13"/>
     </row>
-    <row r="53" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="53" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B53" s="13"/>
       <c r="C53" s="13"/>
       <c r="D53" s="13"/>
@@ -3566,7 +3566,7 @@
       <c r="Q53" s="13"/>
       <c r="R53" s="13"/>
     </row>
-    <row r="54" spans="2:18" x14ac:dyDescent="0.3">
+    <row r="54" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B54" s="13"/>
       <c r="C54" s="13"/>
       <c r="D54" s="13"/>
@@ -3617,17 +3617,17 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7054496A-AF4B-4EC1-B368-49C550220A1C}">
   <sheetPr filterMode="1"/>
   <dimension ref="A1:L301"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="94.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="94.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="16" style="2" customWidth="1"/>
     <col min="5" max="12" width="18" style="2" customWidth="1"/>
     <col min="13" max="13" width="12" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.109375" style="2"/>
+    <col min="14" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3665,7 +3665,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="41" t="s">
         <v>12</v>
       </c>
@@ -3683,7 +3683,7 @@
       <c r="K2" s="6"/>
       <c r="L2" s="6"/>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="41" t="s">
         <v>12</v>
       </c>
@@ -3721,7 +3721,7 @@
         <v>26819200.996155463</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="41" t="s">
         <v>12</v>
       </c>
@@ -3759,7 +3759,7 @@
         <v>56018232.597976193</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="41" t="s">
         <v>12</v>
       </c>
@@ -3797,7 +3797,7 @@
         <v>170565705.92964286</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="41" t="s">
         <v>12</v>
       </c>
@@ -3835,7 +3835,7 @@
         <v>79877180.657261893</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="41" t="s">
         <v>18</v>
       </c>
@@ -3865,7 +3865,7 @@
       <c r="K7" s="6"/>
       <c r="L7" s="6"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="41" t="s">
         <v>18</v>
       </c>
@@ -3895,7 +3895,7 @@
       <c r="K8" s="6"/>
       <c r="L8" s="6"/>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="41" t="s">
         <v>18</v>
       </c>
@@ -3925,7 +3925,7 @@
       <c r="K9" s="6"/>
       <c r="L9" s="6"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="41" t="s">
         <v>18</v>
       </c>
@@ -3955,7 +3955,7 @@
       <c r="K10" s="6"/>
       <c r="L10" s="6"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="41" t="s">
         <v>19</v>
       </c>
@@ -3993,7 +3993,7 @@
         <v>1403270410.0475006</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="41" t="s">
         <v>19</v>
       </c>
@@ -4031,7 +4031,7 @@
         <v>43232783.299999997</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="41" t="s">
         <v>19</v>
       </c>
@@ -4069,7 +4069,7 @@
         <v>789204932.27500033</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="41" t="s">
         <v>19</v>
       </c>
@@ -4107,7 +4107,7 @@
         <v>500814543.58749998</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>20</v>
       </c>
@@ -4125,7 +4125,7 @@
       <c r="K15" s="6"/>
       <c r="L15" s="6"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>21</v>
       </c>
@@ -4143,7 +4143,7 @@
       <c r="K16" s="6"/>
       <c r="L16" s="6"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="41" t="s">
         <v>22</v>
       </c>
@@ -4161,7 +4161,7 @@
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="41" t="s">
         <v>22</v>
       </c>
@@ -4199,7 +4199,7 @@
         <v>12788293.736842105</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="41" t="s">
         <v>22</v>
       </c>
@@ -4237,7 +4237,7 @@
         <v>863986.71500000008</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="41" t="s">
         <v>22</v>
       </c>
@@ -4275,7 +4275,7 @@
         <v>5370201.9115789467</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A21" s="41" t="s">
         <v>22</v>
       </c>
@@ -4313,7 +4313,7 @@
         <v>4313357.7878842624</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A22" s="41" t="s">
         <v>23</v>
       </c>
@@ -4331,7 +4331,7 @@
       <c r="K22" s="6"/>
       <c r="L22" s="6"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A23" s="41" t="s">
         <v>23</v>
       </c>
@@ -4369,7 +4369,7 @@
         <v>44326790.909789473</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="41" t="s">
         <v>23</v>
       </c>
@@ -4387,7 +4387,7 @@
       <c r="K24" s="6"/>
       <c r="L24" s="6"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="41" t="s">
         <v>23</v>
       </c>
@@ -4417,7 +4417,7 @@
       <c r="K25" s="6"/>
       <c r="L25" s="6"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="41" t="s">
         <v>23</v>
       </c>
@@ -4455,7 +4455,7 @@
         <v>430931.20894736843</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>24</v>
       </c>
@@ -4473,7 +4473,7 @@
       <c r="K27" s="6"/>
       <c r="L27" s="6"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="41" t="s">
         <v>25</v>
       </c>
@@ -4511,7 +4511,7 @@
         <v>24359.106315789475</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="41" t="s">
         <v>25</v>
       </c>
@@ -4541,7 +4541,7 @@
       <c r="K29" s="6"/>
       <c r="L29" s="6"/>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="41" t="s">
         <v>25</v>
       </c>
@@ -4567,7 +4567,7 @@
         <v>29653.105263157893</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="41" t="s">
         <v>26</v>
       </c>
@@ -4605,7 +4605,7 @@
         <v>22700002.013999999</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="41" t="s">
         <v>26</v>
       </c>
@@ -4631,7 +4631,7 @@
       <c r="K32" s="6"/>
       <c r="L32" s="6"/>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A33" s="41" t="s">
         <v>26</v>
       </c>
@@ -4669,7 +4669,7 @@
         <v>9708542.1121710539</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="41" t="s">
         <v>27</v>
       </c>
@@ -4707,7 +4707,7 @@
         <v>2385352.0408421056</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A35" s="41" t="s">
         <v>27</v>
       </c>
@@ -4737,7 +4737,7 @@
       <c r="K35" s="6"/>
       <c r="L35" s="6"/>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A36" s="41" t="s">
         <v>27</v>
       </c>
@@ -4763,7 +4763,7 @@
         <v>6987.9032894736847</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A37" s="41" t="s">
         <v>28</v>
       </c>
@@ -4801,7 +4801,7 @@
         <v>3753257.1406578948</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A38" s="41" t="s">
         <v>28</v>
       </c>
@@ -4827,7 +4827,7 @@
       <c r="K38" s="6"/>
       <c r="L38" s="6"/>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A39" s="41" t="s">
         <v>29</v>
       </c>
@@ -4865,7 +4865,7 @@
         <v>17711618.430631582</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A40" s="41" t="s">
         <v>29</v>
       </c>
@@ -4891,7 +4891,7 @@
       <c r="K40" s="6"/>
       <c r="L40" s="6"/>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A41" s="41" t="s">
         <v>29</v>
       </c>
@@ -4929,7 +4929,7 @@
         <v>8274488.3427631576</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A42" s="41" t="s">
         <v>30</v>
       </c>
@@ -4967,7 +4967,7 @@
         <v>12708293.497763159</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A43" s="41" t="s">
         <v>30</v>
       </c>
@@ -4985,7 +4985,7 @@
       <c r="K43" s="6"/>
       <c r="L43" s="6"/>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A44" s="41" t="s">
         <v>30</v>
       </c>
@@ -5023,7 +5023,7 @@
         <v>129709.70407894738</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A45" s="41" t="s">
         <v>31</v>
       </c>
@@ -5041,7 +5041,7 @@
       <c r="K45" s="6"/>
       <c r="L45" s="6"/>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A46" s="41" t="s">
         <v>31</v>
       </c>
@@ -5079,7 +5079,7 @@
         <v>4366498.504999999</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A47" s="41" t="s">
         <v>31</v>
       </c>
@@ -5117,7 +5117,7 @@
         <v>924903.77499999991</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A48" s="41" t="s">
         <v>31</v>
       </c>
@@ -5155,7 +5155,7 @@
         <v>56671594.19749999</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="41" t="s">
         <v>31</v>
       </c>
@@ -5193,7 +5193,7 @@
         <v>28451376.886823118</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" s="41" t="s">
         <v>32</v>
       </c>
@@ -5211,7 +5211,7 @@
       <c r="K50" s="6"/>
       <c r="L50" s="6"/>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="41" t="s">
         <v>32</v>
       </c>
@@ -5229,7 +5229,7 @@
       <c r="K51" s="6"/>
       <c r="L51" s="6"/>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="41" t="s">
         <v>32</v>
       </c>
@@ -5247,7 +5247,7 @@
       <c r="K52" s="6"/>
       <c r="L52" s="6"/>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" s="41" t="s">
         <v>32</v>
       </c>
@@ -5285,7 +5285,7 @@
         <v>1371371.7111111111</v>
       </c>
     </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A54" s="41" t="s">
         <v>33</v>
       </c>
@@ -5323,7 +5323,7 @@
         <v>4588112.7602708973</v>
       </c>
     </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" s="41" t="s">
         <v>33</v>
       </c>
@@ -5361,7 +5361,7 @@
         <v>68258991.188157901</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="41" t="s">
         <v>33</v>
       </c>
@@ -5399,7 +5399,7 @@
         <v>202310628.16776317</v>
       </c>
     </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="41" t="s">
         <v>33</v>
       </c>
@@ -5437,7 +5437,7 @@
         <v>61534344.793815792</v>
       </c>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" s="41" t="s">
         <v>34</v>
       </c>
@@ -5475,7 +5475,7 @@
         <v>99151.439999999988</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" s="41" t="s">
         <v>34</v>
       </c>
@@ -5513,7 +5513,7 @@
         <v>3781590.8850000007</v>
       </c>
     </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" s="41" t="s">
         <v>34</v>
       </c>
@@ -5551,7 +5551,7 @@
         <v>2364272.5157894739</v>
       </c>
     </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A61" s="41" t="s">
         <v>34</v>
       </c>
@@ -5571,7 +5571,7 @@
       <c r="K61" s="6"/>
       <c r="L61" s="6"/>
     </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" s="41" t="s">
         <v>35</v>
       </c>
@@ -5609,7 +5609,7 @@
         <v>42709218.048947372</v>
       </c>
     </row>
-    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A63" s="41" t="s">
         <v>35</v>
       </c>
@@ -5647,7 +5647,7 @@
         <v>585519.70234210533</v>
       </c>
     </row>
-    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A64" s="41" t="s">
         <v>35</v>
       </c>
@@ -5685,7 +5685,7 @@
         <v>6391844.9436842091</v>
       </c>
     </row>
-    <row r="65" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A65" s="41" t="s">
         <v>36</v>
       </c>
@@ -5703,7 +5703,7 @@
       <c r="K65" s="6"/>
       <c r="L65" s="6"/>
     </row>
-    <row r="66" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A66" s="41" t="s">
         <v>36</v>
       </c>
@@ -5741,7 +5741,7 @@
         <v>71135570.336828187</v>
       </c>
     </row>
-    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A67" s="41" t="s">
         <v>36</v>
       </c>
@@ -5779,7 +5779,7 @@
         <v>8918362.7869736832</v>
       </c>
     </row>
-    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A68" s="41" t="s">
         <v>36</v>
       </c>
@@ -5817,7 +5817,7 @@
         <v>56037443.403815791</v>
       </c>
     </row>
-    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A69" s="41" t="s">
         <v>36</v>
       </c>
@@ -5855,7 +5855,7 @@
         <v>26078721.471578948</v>
       </c>
     </row>
-    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A70" s="41" t="s">
         <v>37</v>
       </c>
@@ -5873,7 +5873,7 @@
       <c r="K70" s="6"/>
       <c r="L70" s="6"/>
     </row>
-    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A71" s="41" t="s">
         <v>37</v>
       </c>
@@ -5911,7 +5911,7 @@
         <v>13285092.037631579</v>
       </c>
     </row>
-    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A72" s="41" t="s">
         <v>37</v>
       </c>
@@ -5929,7 +5929,7 @@
       <c r="K72" s="6"/>
       <c r="L72" s="6"/>
     </row>
-    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A73" s="41" t="s">
         <v>37</v>
       </c>
@@ -5959,7 +5959,7 @@
       <c r="K73" s="6"/>
       <c r="L73" s="6"/>
     </row>
-    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A74" s="41" t="s">
         <v>37</v>
       </c>
@@ -5997,7 +5997,7 @@
         <v>7212690.1784210531</v>
       </c>
     </row>
-    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A75" s="41" t="s">
         <v>38</v>
       </c>
@@ -6027,7 +6027,7 @@
         <v>3143161.6294736844</v>
       </c>
     </row>
-    <row r="76" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A76" s="41" t="s">
         <v>38</v>
       </c>
@@ -6053,7 +6053,7 @@
       <c r="K76" s="6"/>
       <c r="L76" s="6"/>
     </row>
-    <row r="77" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>39</v>
       </c>
@@ -6091,7 +6091,7 @@
         <v>694846.97368421056</v>
       </c>
     </row>
-    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A78" s="41" t="s">
         <v>40</v>
       </c>
@@ -6129,7 +6129,7 @@
         <v>31169164.653893046</v>
       </c>
     </row>
-    <row r="79" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A79" s="41" t="s">
         <v>40</v>
       </c>
@@ -6167,7 +6167,7 @@
         <v>9024207.2250826061</v>
       </c>
     </row>
-    <row r="80" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A80" s="41" t="s">
         <v>40</v>
       </c>
@@ -6205,7 +6205,7 @@
         <v>26014337.772836529</v>
       </c>
     </row>
-    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A81" s="41" t="s">
         <v>40</v>
       </c>
@@ -6243,7 +6243,7 @@
         <v>21218834.523721006</v>
       </c>
     </row>
-    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A82" s="41" t="s">
         <v>41</v>
       </c>
@@ -6281,7 +6281,7 @@
         <v>24485113.215146199</v>
       </c>
     </row>
-    <row r="83" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A83" s="41" t="s">
         <v>41</v>
       </c>
@@ -6319,7 +6319,7 @@
         <v>42986086.185204685</v>
       </c>
     </row>
-    <row r="84" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A84" s="41" t="s">
         <v>41</v>
       </c>
@@ -6357,7 +6357,7 @@
         <v>89969889.638869569</v>
       </c>
     </row>
-    <row r="85" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A85" s="41" t="s">
         <v>41</v>
       </c>
@@ -6395,7 +6395,7 @@
         <v>43092807.72445029</v>
       </c>
     </row>
-    <row r="86" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A86" s="41" t="s">
         <v>42</v>
       </c>
@@ -6433,7 +6433,7 @@
         <v>26223826.190433443</v>
       </c>
     </row>
-    <row r="87" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A87" s="41" t="s">
         <v>42</v>
       </c>
@@ -6451,7 +6451,7 @@
       <c r="K87" s="6"/>
       <c r="L87" s="6"/>
     </row>
-    <row r="88" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A88" s="41" t="s">
         <v>42</v>
       </c>
@@ -6489,7 +6489,7 @@
         <v>38913109.206510134</v>
       </c>
     </row>
-    <row r="89" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A89" s="41" t="s">
         <v>42</v>
       </c>
@@ -6527,7 +6527,7 @@
         <v>8318128.2670879252</v>
       </c>
     </row>
-    <row r="90" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A90" s="42" t="s">
         <v>43</v>
       </c>
@@ -6545,7 +6545,7 @@
       <c r="K90" s="6"/>
       <c r="L90" s="6"/>
     </row>
-    <row r="91" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A91" s="43" t="s">
         <v>43</v>
       </c>
@@ -6583,7 +6583,7 @@
         <v>593298.1894736843</v>
       </c>
     </row>
-    <row r="92" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A92" s="43" t="s">
         <v>43</v>
       </c>
@@ -6621,7 +6621,7 @@
         <v>882693.01642857143</v>
       </c>
     </row>
-    <row r="93" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A93" s="43" t="s">
         <v>43</v>
       </c>
@@ -6659,7 +6659,7 @@
         <v>68866.200000000012</v>
       </c>
     </row>
-    <row r="94" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A94" s="44" t="s">
         <v>43</v>
       </c>
@@ -6697,7 +6697,7 @@
         <v>9727462.9341666661</v>
       </c>
     </row>
-    <row r="95" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A95" s="41" t="s">
         <v>44</v>
       </c>
@@ -6735,7 +6735,7 @@
         <v>500000</v>
       </c>
     </row>
-    <row r="96" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A96" s="41" t="s">
         <v>44</v>
       </c>
@@ -6773,7 +6773,7 @@
         <v>16995032.578833334</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A97" s="41" t="s">
         <v>44</v>
       </c>
@@ -6811,7 +6811,7 @@
         <v>22529845.132500004</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A98" s="41" t="s">
         <v>45</v>
       </c>
@@ -6841,7 +6841,7 @@
         <v>11652763.552941177</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A99" s="41" t="s">
         <v>45</v>
       </c>
@@ -6859,7 +6859,7 @@
       <c r="K99" s="6"/>
       <c r="L99" s="6"/>
     </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A100" s="41" t="s">
         <v>45</v>
       </c>
@@ -6885,7 +6885,7 @@
       <c r="K100" s="6"/>
       <c r="L100" s="6"/>
     </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A101" s="41" t="s">
         <v>46</v>
       </c>
@@ -6923,7 +6923,7 @@
         <v>3129137.4496973683</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A102" s="41" t="s">
         <v>46</v>
       </c>
@@ -6941,7 +6941,7 @@
       <c r="K102" s="6"/>
       <c r="L102" s="6"/>
     </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A103" s="41" t="s">
         <v>46</v>
       </c>
@@ -6967,7 +6967,7 @@
       <c r="K103" s="6"/>
       <c r="L103" s="6"/>
     </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A104" s="41" t="s">
         <v>47</v>
       </c>
@@ -6997,7 +6997,7 @@
         <v>19439134.578947369</v>
       </c>
     </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A105" s="41" t="s">
         <v>47</v>
       </c>
@@ -7025,7 +7025,7 @@
       <c r="K105" s="6"/>
       <c r="L105" s="6"/>
     </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A106" s="41" t="s">
         <v>47</v>
       </c>
@@ -7061,7 +7061,7 @@
         <v>12278482.1775</v>
       </c>
     </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A107" s="41" t="s">
         <v>48</v>
       </c>
@@ -7099,7 +7099,7 @@
         <v>600000</v>
       </c>
     </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A108" s="41" t="s">
         <v>48</v>
       </c>
@@ -7137,7 +7137,7 @@
         <v>428081.60342105263</v>
       </c>
     </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A109" s="41" t="s">
         <v>48</v>
       </c>
@@ -7155,7 +7155,7 @@
       <c r="K109" s="6"/>
       <c r="L109" s="6"/>
     </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A110" s="41" t="s">
         <v>49</v>
       </c>
@@ -7193,7 +7193,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A111" s="41" t="s">
         <v>49</v>
       </c>
@@ -7231,7 +7231,7 @@
         <v>15938780.685739476</v>
       </c>
     </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A112" s="41" t="s">
         <v>49</v>
       </c>
@@ -7267,7 +7267,7 @@
         <v>7463.7629999999999</v>
       </c>
     </row>
-    <row r="113" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A113" s="41" t="s">
         <v>49</v>
       </c>
@@ -7305,7 +7305,7 @@
         <v>6024488.8079210529</v>
       </c>
     </row>
-    <row r="114" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A114" s="41" t="s">
         <v>50</v>
       </c>
@@ -7343,7 +7343,7 @@
         <v>540000</v>
       </c>
     </row>
-    <row r="115" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A115" s="41" t="s">
         <v>50</v>
       </c>
@@ -7381,7 +7381,7 @@
         <v>3357564.5291447369</v>
       </c>
     </row>
-    <row r="116" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A116" s="41" t="s">
         <v>50</v>
       </c>
@@ -7419,7 +7419,7 @@
         <v>277375.88714868418</v>
       </c>
     </row>
-    <row r="117" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A117" s="41" t="s">
         <v>50</v>
       </c>
@@ -7457,7 +7457,7 @@
         <v>48463.652665350877</v>
       </c>
     </row>
-    <row r="118" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A118" s="41" t="s">
         <v>50</v>
       </c>
@@ -7493,7 +7493,7 @@
         <v>962589.57300000009</v>
       </c>
     </row>
-    <row r="119" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="s">
         <v>51</v>
       </c>
@@ -7531,7 +7531,7 @@
         <v>4199871.1182460524</v>
       </c>
     </row>
-    <row r="120" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A120" s="41" t="s">
         <v>52</v>
       </c>
@@ -7549,7 +7549,7 @@
       <c r="K120" s="6"/>
       <c r="L120" s="6"/>
     </row>
-    <row r="121" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A121" s="41" t="s">
         <v>52</v>
       </c>
@@ -7581,7 +7581,7 @@
         <v>8001.5255263157915</v>
       </c>
     </row>
-    <row r="122" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A122" s="41" t="s">
         <v>52</v>
       </c>
@@ -7619,7 +7619,7 @@
         <v>196251.34736842106</v>
       </c>
     </row>
-    <row r="123" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A123" s="41" t="s">
         <v>53</v>
       </c>
@@ -7657,7 +7657,7 @@
         <v>300000</v>
       </c>
     </row>
-    <row r="124" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A124" s="41" t="s">
         <v>53</v>
       </c>
@@ -7695,7 +7695,7 @@
         <v>3969424.3796421057</v>
       </c>
     </row>
-    <row r="125" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A125" s="41" t="s">
         <v>53</v>
       </c>
@@ -7733,7 +7733,7 @@
         <v>8895367.3138157893</v>
       </c>
     </row>
-    <row r="126" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A126" s="41" t="s">
         <v>54</v>
       </c>
@@ -7751,7 +7751,7 @@
       <c r="K126" s="6"/>
       <c r="L126" s="6"/>
     </row>
-    <row r="127" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A127" s="41" t="s">
         <v>54</v>
       </c>
@@ -7769,7 +7769,7 @@
       <c r="K127" s="6"/>
       <c r="L127" s="6"/>
     </row>
-    <row r="128" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A128" s="41" t="s">
         <v>54</v>
       </c>
@@ -7787,7 +7787,7 @@
       <c r="K128" s="6"/>
       <c r="L128" s="6"/>
     </row>
-    <row r="129" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A129" s="41" t="s">
         <v>54</v>
       </c>
@@ -7807,7 +7807,7 @@
       <c r="K129" s="6"/>
       <c r="L129" s="6"/>
     </row>
-    <row r="130" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A130" s="41" t="s">
         <v>55</v>
       </c>
@@ -7825,7 +7825,7 @@
       <c r="K130" s="6"/>
       <c r="L130" s="6"/>
     </row>
-    <row r="131" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A131" s="41" t="s">
         <v>55</v>
       </c>
@@ -7863,7 +7863,7 @@
         <v>44666553.82686425</v>
       </c>
     </row>
-    <row r="132" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A132" s="41" t="s">
         <v>55</v>
       </c>
@@ -7901,7 +7901,7 @@
         <v>2148068.0935714287</v>
       </c>
     </row>
-    <row r="133" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A133" s="41" t="s">
         <v>55</v>
       </c>
@@ -7939,7 +7939,7 @@
         <v>10829590.64130117</v>
       </c>
     </row>
-    <row r="134" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A134" s="41" t="s">
         <v>55</v>
       </c>
@@ -7977,7 +7977,7 @@
         <v>53816727.563368849</v>
       </c>
     </row>
-    <row r="135" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A135" s="41" t="s">
         <v>56</v>
       </c>
@@ -8015,7 +8015,7 @@
         <v>5366204.9252105262</v>
       </c>
     </row>
-    <row r="136" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A136" s="41" t="s">
         <v>56</v>
       </c>
@@ -8053,7 +8053,7 @@
         <v>1918456.0949999997</v>
       </c>
     </row>
-    <row r="137" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A137" s="41" t="s">
         <v>57</v>
       </c>
@@ -8091,7 +8091,7 @@
         <v>2456094.4891353385</v>
       </c>
     </row>
-    <row r="138" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A138" s="41" t="s">
         <v>57</v>
       </c>
@@ -8129,7 +8129,7 @@
         <v>84871745.658650786</v>
       </c>
     </row>
-    <row r="139" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A139" s="41" t="s">
         <v>57</v>
       </c>
@@ -8167,7 +8167,7 @@
         <v>228007209.74936509</v>
       </c>
     </row>
-    <row r="140" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A140" s="41" t="s">
         <v>57</v>
       </c>
@@ -8205,7 +8205,7 @@
         <v>32273220.97396826</v>
       </c>
     </row>
-    <row r="141" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A141" s="3" t="s">
         <v>58</v>
       </c>
@@ -8243,7 +8243,7 @@
         <v>1012182.5810526316</v>
       </c>
     </row>
-    <row r="142" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A142" s="41" t="s">
         <v>59</v>
       </c>
@@ -8281,7 +8281,7 @@
         <v>4000000</v>
       </c>
     </row>
-    <row r="143" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A143" s="41" t="s">
         <v>59</v>
       </c>
@@ -8319,7 +8319,7 @@
         <v>19377207.360228568</v>
       </c>
     </row>
-    <row r="144" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A144" s="41" t="s">
         <v>59</v>
       </c>
@@ -8357,7 +8357,7 @@
         <v>123225959.44543454</v>
       </c>
     </row>
-    <row r="145" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A145" s="41" t="s">
         <v>59</v>
       </c>
@@ -8385,7 +8385,7 @@
         <v>9816494.2557882406</v>
       </c>
     </row>
-    <row r="146" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A146" s="41" t="s">
         <v>60</v>
       </c>
@@ -8423,7 +8423,7 @@
         <v>85488520.6669323</v>
       </c>
     </row>
-    <row r="147" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A147" s="41" t="s">
         <v>60</v>
       </c>
@@ -8461,7 +8461,7 @@
         <v>57292565.508875743</v>
       </c>
     </row>
-    <row r="148" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A148" s="41" t="s">
         <v>60</v>
       </c>
@@ -8499,7 +8499,7 @@
         <v>162941685.62800577</v>
       </c>
     </row>
-    <row r="149" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A149" s="41" t="s">
         <v>60</v>
       </c>
@@ -8537,7 +8537,7 @@
         <v>66591452.998300254</v>
       </c>
     </row>
-    <row r="150" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A150" s="41" t="s">
         <v>61</v>
       </c>
@@ -8575,7 +8575,7 @@
         <v>6418700.4964842089</v>
       </c>
     </row>
-    <row r="151" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A151" s="41" t="s">
         <v>61</v>
       </c>
@@ -8613,7 +8613,7 @@
         <v>657.72019736842117</v>
       </c>
     </row>
-    <row r="152" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A152" s="41" t="s">
         <v>61</v>
       </c>
@@ -8651,7 +8651,7 @@
         <v>38980.994268421055</v>
       </c>
     </row>
-    <row r="153" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A153" s="41" t="s">
         <v>62</v>
       </c>
@@ -8689,7 +8689,7 @@
         <v>57668115.752105266</v>
       </c>
     </row>
-    <row r="154" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A154" s="41" t="s">
         <v>62</v>
       </c>
@@ -8727,7 +8727,7 @@
         <v>48207996.665438592</v>
       </c>
     </row>
-    <row r="155" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A155" s="41" t="s">
         <v>62</v>
       </c>
@@ -8765,7 +8765,7 @@
         <v>163594841.15653506</v>
       </c>
     </row>
-    <row r="156" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A156" s="41" t="s">
         <v>62</v>
       </c>
@@ -8803,7 +8803,7 @@
         <v>51145121.535921052</v>
       </c>
     </row>
-    <row r="157" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A157" s="41" t="s">
         <v>63</v>
       </c>
@@ -8829,7 +8829,7 @@
         <v>1140116.518780523</v>
       </c>
     </row>
-    <row r="158" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A158" s="41" t="s">
         <v>63</v>
       </c>
@@ -8855,7 +8855,7 @@
         <v>3095533.6346984911</v>
       </c>
     </row>
-    <row r="159" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A159" s="41" t="s">
         <v>63</v>
       </c>
@@ -8883,7 +8883,7 @@
         <v>24073104.668296658</v>
       </c>
     </row>
-    <row r="160" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A160" s="41" t="s">
         <v>63</v>
       </c>
@@ -8911,7 +8911,7 @@
         <v>8249515.7360912031</v>
       </c>
     </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A161" s="41" t="s">
         <v>64</v>
       </c>
@@ -8929,7 +8929,7 @@
       <c r="K161" s="6"/>
       <c r="L161" s="6"/>
     </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A162" s="41" t="s">
         <v>64</v>
       </c>
@@ -8947,7 +8947,7 @@
       <c r="K162" s="6"/>
       <c r="L162" s="6"/>
     </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A163" s="41" t="s">
         <v>64</v>
       </c>
@@ -8967,7 +8967,7 @@
       <c r="K163" s="6"/>
       <c r="L163" s="6"/>
     </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A164" s="41" t="s">
         <v>65</v>
       </c>
@@ -8995,7 +8995,7 @@
         <v>524620.18888888881</v>
       </c>
     </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A165" s="41" t="s">
         <v>65</v>
       </c>
@@ -9033,7 +9033,7 @@
         <v>11686619.239444446</v>
       </c>
     </row>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A166" s="41" t="s">
         <v>65</v>
       </c>
@@ -9071,7 +9071,7 @@
         <v>67230835.707277775</v>
       </c>
     </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A167" s="41" t="s">
         <v>65</v>
       </c>
@@ -9109,7 +9109,7 @@
         <v>8927850.3513888884</v>
       </c>
     </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A168" s="41" t="s">
         <v>66</v>
       </c>
@@ -9127,7 +9127,7 @@
       <c r="K168" s="6"/>
       <c r="L168" s="6"/>
     </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A169" s="41" t="s">
         <v>66</v>
       </c>
@@ -9165,7 +9165,7 @@
         <v>11586096.10842105</v>
       </c>
     </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A170" s="41" t="s">
         <v>66</v>
       </c>
@@ -9203,7 +9203,7 @@
         <v>61286058.379432946</v>
       </c>
     </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A171" s="41" t="s">
         <v>66</v>
       </c>
@@ -9241,7 +9241,7 @@
         <v>198326735.48209769</v>
       </c>
     </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A172" s="41" t="s">
         <v>66</v>
       </c>
@@ -9279,7 +9279,7 @@
         <v>74368544.324421823</v>
       </c>
     </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A173" s="41" t="s">
         <v>67</v>
       </c>
@@ -9317,7 +9317,7 @@
         <v>37434.968421052632</v>
       </c>
     </row>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A174" s="41" t="s">
         <v>67</v>
       </c>
@@ -9335,7 +9335,7 @@
       <c r="K174" s="6"/>
       <c r="L174" s="6"/>
     </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A175" s="41" t="s">
         <v>67</v>
       </c>
@@ -9353,7 +9353,7 @@
       <c r="K175" s="6"/>
       <c r="L175" s="6"/>
     </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A176" s="41" t="s">
         <v>68</v>
       </c>
@@ -9391,7 +9391,7 @@
         <v>14085732.501447368</v>
       </c>
     </row>
-    <row r="177" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A177" s="41" t="s">
         <v>68</v>
       </c>
@@ -9423,7 +9423,7 @@
       <c r="K177" s="6"/>
       <c r="L177" s="6"/>
     </row>
-    <row r="178" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A178" s="41" t="s">
         <v>68</v>
       </c>
@@ -9461,7 +9461,7 @@
         <v>2658726.6143421056</v>
       </c>
     </row>
-    <row r="179" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A179" s="41" t="s">
         <v>69</v>
       </c>
@@ -9499,7 +9499,7 @@
         <v>5274066.9230263159</v>
       </c>
     </row>
-    <row r="180" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A180" s="41" t="s">
         <v>69</v>
       </c>
@@ -9525,7 +9525,7 @@
       <c r="K180" s="6"/>
       <c r="L180" s="6"/>
     </row>
-    <row r="181" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A181" s="41" t="s">
         <v>69</v>
       </c>
@@ -9563,7 +9563,7 @@
         <v>109338.78881578946</v>
       </c>
     </row>
-    <row r="182" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A182" s="41" t="s">
         <v>70</v>
       </c>
@@ -9581,7 +9581,7 @@
       <c r="K182" s="6"/>
       <c r="L182" s="6"/>
     </row>
-    <row r="183" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A183" s="41" t="s">
         <v>70</v>
       </c>
@@ -9599,7 +9599,7 @@
       <c r="K183" s="6"/>
       <c r="L183" s="6"/>
     </row>
-    <row r="184" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A184" s="41" t="s">
         <v>70</v>
       </c>
@@ -9617,7 +9617,7 @@
       <c r="K184" s="6"/>
       <c r="L184" s="6"/>
     </row>
-    <row r="185" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A185" s="41" t="s">
         <v>70</v>
       </c>
@@ -9635,7 +9635,7 @@
       <c r="K185" s="6"/>
       <c r="L185" s="6"/>
     </row>
-    <row r="186" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A186" s="41" t="s">
         <v>70</v>
       </c>
@@ -9653,7 +9653,7 @@
       <c r="K186" s="6"/>
       <c r="L186" s="6"/>
     </row>
-    <row r="187" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A187" s="41" t="s">
         <v>71</v>
       </c>
@@ -9671,7 +9671,7 @@
       <c r="K187" s="6"/>
       <c r="L187" s="6"/>
     </row>
-    <row r="188" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A188" s="41" t="s">
         <v>71</v>
       </c>
@@ -9709,7 +9709,7 @@
         <v>1602020.15372807</v>
       </c>
     </row>
-    <row r="189" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A189" s="41" t="s">
         <v>71</v>
       </c>
@@ -9747,7 +9747,7 @@
         <v>3089470.1716666664</v>
       </c>
     </row>
-    <row r="190" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A190" s="41" t="s">
         <v>71</v>
       </c>
@@ -9773,7 +9773,7 @@
       <c r="K190" s="6"/>
       <c r="L190" s="6"/>
     </row>
-    <row r="191" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A191" s="41" t="s">
         <v>71</v>
       </c>
@@ -9811,7 +9811,7 @@
         <v>8435990.8228508774</v>
       </c>
     </row>
-    <row r="192" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A192" s="41" t="s">
         <v>72</v>
       </c>
@@ -9829,7 +9829,7 @@
       <c r="K192" s="6"/>
       <c r="L192" s="6"/>
     </row>
-    <row r="193" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A193" s="41" t="s">
         <v>72</v>
       </c>
@@ -9867,7 +9867,7 @@
         <v>41053.861588892236</v>
       </c>
     </row>
-    <row r="194" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A194" s="41" t="s">
         <v>72</v>
       </c>
@@ -9897,7 +9897,7 @@
       <c r="K194" s="6"/>
       <c r="L194" s="6"/>
     </row>
-    <row r="195" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A195" s="41" t="s">
         <v>72</v>
       </c>
@@ -9935,7 +9935,7 @@
         <v>361138.98097679514</v>
       </c>
     </row>
-    <row r="196" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A196" s="41" t="s">
         <v>73</v>
       </c>
@@ -9973,7 +9973,7 @@
         <v>21801576.347789474</v>
       </c>
     </row>
-    <row r="197" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A197" s="41" t="s">
         <v>73</v>
       </c>
@@ -9991,7 +9991,7 @@
       <c r="K197" s="6"/>
       <c r="L197" s="6"/>
     </row>
-    <row r="198" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A198" s="41" t="s">
         <v>73</v>
       </c>
@@ -10029,7 +10029,7 @@
         <v>4773371.973289473</v>
       </c>
     </row>
-    <row r="199" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A199" s="41" t="s">
         <v>74</v>
       </c>
@@ -10067,7 +10067,7 @@
         <v>6000000</v>
       </c>
     </row>
-    <row r="200" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A200" s="41" t="s">
         <v>74</v>
       </c>
@@ -10105,7 +10105,7 @@
         <v>95686.964999999997</v>
       </c>
     </row>
-    <row r="201" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A201" s="41" t="s">
         <v>74</v>
       </c>
@@ -10143,7 +10143,7 @@
         <v>19427327.223125003</v>
       </c>
     </row>
-    <row r="202" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A202" s="41" t="s">
         <v>74</v>
       </c>
@@ -10181,7 +10181,7 @@
         <v>28291617.551274512</v>
       </c>
     </row>
-    <row r="203" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A203" s="41" t="s">
         <v>74</v>
       </c>
@@ -10219,7 +10219,7 @@
         <v>21470697.767319441</v>
       </c>
     </row>
-    <row r="204" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C204" s="8"/>
       <c r="D204" s="8"/>
       <c r="E204" s="8"/>
@@ -10231,7 +10231,7 @@
       <c r="K204" s="8"/>
       <c r="L204" s="8"/>
     </row>
-    <row r="205" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C205" s="8"/>
       <c r="D205" s="8"/>
       <c r="E205" s="8"/>
@@ -10243,7 +10243,7 @@
       <c r="K205" s="8"/>
       <c r="L205" s="8"/>
     </row>
-    <row r="206" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C206" s="8"/>
       <c r="D206" s="8"/>
       <c r="E206" s="8"/>
@@ -10255,7 +10255,7 @@
       <c r="K206" s="8"/>
       <c r="L206" s="8"/>
     </row>
-    <row r="207" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A207" s="2" t="s">
         <v>43</v>
       </c>
@@ -10303,7 +10303,7 @@
         <v>22913488.673833333</v>
       </c>
     </row>
-    <row r="208" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A208" s="2" t="s">
         <v>57</v>
       </c>
@@ -10351,7 +10351,7 @@
         <v>312878955.40801585</v>
       </c>
     </row>
-    <row r="209" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A209" s="2" t="s">
         <v>55</v>
       </c>
@@ -10399,7 +10399,7 @@
         <v>12977658.734872598</v>
       </c>
     </row>
-    <row r="210" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A210" s="2" t="s">
         <v>71</v>
       </c>
@@ -10447,7 +10447,7 @@
         <v>3089470.1716666664</v>
       </c>
     </row>
-    <row r="211" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A211" s="2" t="s">
         <v>66</v>
       </c>
@@ -10495,7 +10495,7 @@
         <v>259612793.86153063</v>
       </c>
     </row>
-    <row r="212" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A212" s="2" t="s">
         <v>108</v>
       </c>
@@ -10543,7 +10543,7 @@
         <v>6234188.6265789466</v>
       </c>
     </row>
-    <row r="213" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A213" s="2" t="s">
         <v>109</v>
       </c>
@@ -10591,7 +10591,7 @@
         <v>57596497.972499989</v>
       </c>
     </row>
-    <row r="214" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A214" s="2" t="s">
         <v>98</v>
       </c>
@@ -10639,7 +10639,7 @@
         <v>6145863.4007894751</v>
       </c>
     </row>
-    <row r="215" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A215" s="2" t="s">
         <v>99</v>
       </c>
@@ -10687,7 +10687,7 @@
         <v>270569619.35592109</v>
       </c>
     </row>
-    <row r="216" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A216" s="16" t="s">
         <v>100</v>
       </c>
@@ -10735,7 +10735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="217" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A217" s="2" t="s">
         <v>101</v>
       </c>
@@ -10783,7 +10783,7 @@
         <v>132955975.82407425</v>
       </c>
     </row>
-    <row r="218" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A218" s="2" t="s">
         <v>102</v>
       </c>
@@ -10831,7 +10831,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="219" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A219" s="2" t="s">
         <v>103</v>
       </c>
@@ -10879,7 +10879,7 @@
         <v>35038544.997919135</v>
       </c>
     </row>
-    <row r="220" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A220" s="2" t="s">
         <v>104</v>
       </c>
@@ -10927,7 +10927,7 @@
         <v>64955806.190789476</v>
       </c>
     </row>
-    <row r="221" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A221" s="2" t="s">
         <v>105</v>
       </c>
@@ -10975,7 +10975,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="222" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A222" s="2" t="s">
         <v>62</v>
       </c>
@@ -11023,7 +11023,7 @@
         <v>211802837.82197365</v>
       </c>
     </row>
-    <row r="223" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A223" s="2" t="s">
         <v>60</v>
       </c>
@@ -11071,10 +11071,10 @@
         <v>220234251.13688153</v>
       </c>
     </row>
-    <row r="224" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C224" s="8"/>
     </row>
-    <row r="225" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A225" s="2" t="s">
         <v>113</v>
       </c>
@@ -11087,7 +11087,7 @@
       <c r="F225" s="8"/>
       <c r="G225" s="8"/>
     </row>
-    <row r="226" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A226" s="2" t="s">
         <v>114</v>
       </c>
@@ -11096,7 +11096,7 @@
       </c>
       <c r="C226" s="8"/>
     </row>
-    <row r="227" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A227" s="2" t="s">
         <v>106</v>
       </c>
@@ -11104,14 +11104,14 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="228" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H228" s="15"/>
       <c r="I228" s="15"/>
       <c r="J228" s="15"/>
       <c r="K228" s="15"/>
       <c r="L228" s="15"/>
     </row>
-    <row r="229" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B229" s="2" t="s">
         <v>115</v>
       </c>
@@ -11121,7 +11121,7 @@
       <c r="K229" s="27"/>
       <c r="L229" s="27"/>
     </row>
-    <row r="230" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A230" s="18" t="s">
         <v>43</v>
       </c>
@@ -11166,7 +11166,7 @@
         <v>20622139.806450002</v>
       </c>
     </row>
-    <row r="231" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A231" s="2" t="s">
         <v>75</v>
       </c>
@@ -11214,7 +11214,7 @@
         <v>16872659.841640912</v>
       </c>
     </row>
-    <row r="232" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A232" s="2" t="s">
         <v>118</v>
       </c>
@@ -11262,7 +11262,7 @@
         <v>3749479.9648090904</v>
       </c>
     </row>
-    <row r="233" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A233" s="18" t="s">
         <v>57</v>
       </c>
@@ -11307,7 +11307,7 @@
         <v>281591059.86721426</v>
       </c>
     </row>
-    <row r="234" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A234" s="2" t="s">
         <v>75</v>
       </c>
@@ -11355,7 +11355,7 @@
         <v>203910767.49005172</v>
       </c>
     </row>
-    <row r="235" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A235" s="2" t="s">
         <v>119</v>
       </c>
@@ -11403,7 +11403,7 @@
         <v>77680292.377162561</v>
       </c>
     </row>
-    <row r="236" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A236" s="18" t="s">
         <v>55</v>
       </c>
@@ -11448,7 +11448,7 @@
         <v>11679892.861385338</v>
       </c>
     </row>
-    <row r="237" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A237" s="2" t="s">
         <v>116</v>
       </c>
@@ -11496,7 +11496,7 @@
         <v>3412103.5325395376</v>
       </c>
     </row>
-    <row r="238" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A238" s="2" t="s">
         <v>117</v>
       </c>
@@ -11544,7 +11544,7 @@
         <v>8267789.3288458008</v>
       </c>
     </row>
-    <row r="239" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A239" s="18" t="s">
         <v>71</v>
       </c>
@@ -11589,7 +11589,7 @@
         <v>3089470.1716666664</v>
       </c>
     </row>
-    <row r="240" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A240" s="2" t="s">
         <v>75</v>
       </c>
@@ -11637,7 +11637,7 @@
         <v>2289842.5978235295</v>
       </c>
     </row>
-    <row r="241" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A241" s="2" t="s">
         <v>118</v>
       </c>
@@ -11685,7 +11685,7 @@
         <v>508853.91062745103</v>
       </c>
     </row>
-    <row r="242" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A242" s="2" t="s">
         <v>81</v>
       </c>
@@ -11733,7 +11733,7 @@
         <v>290773.66321568622</v>
       </c>
     </row>
-    <row r="243" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A243" s="18" t="s">
         <v>66</v>
       </c>
@@ -11778,7 +11778,7 @@
         <v>259612793.86153063</v>
       </c>
     </row>
-    <row r="244" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A244" s="2" t="s">
         <v>75</v>
       </c>
@@ -11826,7 +11826,7 @@
         <v>192418894.27384037</v>
       </c>
     </row>
-    <row r="245" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A245" s="2" t="s">
         <v>118</v>
       </c>
@@ -11874,7 +11874,7 @@
         <v>42759754.283075638</v>
       </c>
     </row>
-    <row r="246" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A246" s="2" t="s">
         <v>81</v>
       </c>
@@ -11922,7 +11922,7 @@
         <v>24434145.304614648</v>
       </c>
     </row>
-    <row r="247" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A247" s="18" t="s">
         <v>108</v>
       </c>
@@ -11967,7 +11967,7 @@
         <v>6857607.4892368419</v>
       </c>
     </row>
-    <row r="248" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A248" s="2" t="s">
         <v>75</v>
       </c>
@@ -12015,7 +12015,7 @@
         <v>5082697.3155520121</v>
       </c>
     </row>
-    <row r="249" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A249" s="2" t="s">
         <v>118</v>
       </c>
@@ -12063,7 +12063,7 @@
         <v>1129488.2923448917</v>
       </c>
     </row>
-    <row r="250" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A250" s="2" t="s">
         <v>81</v>
       </c>
@@ -12111,7 +12111,7 @@
         <v>645421.88133993803</v>
       </c>
     </row>
-    <row r="251" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A251" s="18" t="s">
         <v>109</v>
       </c>
@@ -12156,7 +12156,7 @@
         <v>63356147.769749992</v>
       </c>
     </row>
-    <row r="252" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A252" s="2" t="s">
         <v>75</v>
       </c>
@@ -12204,7 +12204,7 @@
         <v>45878589.764301717</v>
       </c>
     </row>
-    <row r="253" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A253" s="2" t="s">
         <v>119</v>
       </c>
@@ -12252,7 +12252,7 @@
         <v>17477558.005448274</v>
       </c>
     </row>
-    <row r="254" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A254" s="18" t="s">
         <v>98</v>
       </c>
@@ -12297,7 +12297,7 @@
         <v>6145863.4007894751</v>
       </c>
     </row>
-    <row r="255" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A255" s="2" t="s">
         <v>75</v>
       </c>
@@ -12345,7 +12345,7 @@
         <v>6145863.4007894751</v>
       </c>
     </row>
-    <row r="256" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A256" s="18" t="s">
         <v>99</v>
       </c>
@@ -12390,7 +12390,7 @@
         <v>297626581.2915132</v>
       </c>
     </row>
-    <row r="257" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A257" s="2" t="s">
         <v>75</v>
       </c>
@@ -12438,7 +12438,7 @@
         <v>165933403.72889677</v>
       </c>
     </row>
-    <row r="258" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A258" s="2" t="s">
         <v>118</v>
       </c>
@@ -12486,7 +12486,7 @@
         <v>36874089.717532612</v>
       </c>
     </row>
-    <row r="259" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A259" s="2" t="s">
         <v>119</v>
       </c>
@@ -12534,7 +12534,7 @@
         <v>63212725.230055898</v>
       </c>
     </row>
-    <row r="260" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A260" s="2" t="s">
         <v>82</v>
       </c>
@@ -12582,7 +12582,7 @@
         <v>21070908.410018638</v>
       </c>
     </row>
-    <row r="261" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A261" s="2" t="s">
         <v>83</v>
       </c>
@@ -12630,12 +12630,12 @@
         <v>10535454.205009319</v>
       </c>
     </row>
-    <row r="262" spans="1:12" s="21" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:12" s="21" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A262" s="23" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="263" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A263" s="18" t="s">
         <v>101</v>
       </c>
@@ -12680,7 +12680,7 @@
         <v>146251573.40648168</v>
       </c>
     </row>
-    <row r="264" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A264" t="s">
         <v>82</v>
       </c>
@@ -12728,7 +12728,7 @@
         <v>53182390.329629704</v>
       </c>
     </row>
-    <row r="265" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A265" t="s">
         <v>84</v>
       </c>
@@ -12776,7 +12776,7 @@
         <v>19943396.373611137</v>
       </c>
     </row>
-    <row r="266" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A266" t="s">
         <v>85</v>
       </c>
@@ -12824,7 +12824,7 @@
         <v>13295597.582407426</v>
       </c>
     </row>
-    <row r="267" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A267" t="s">
         <v>86</v>
       </c>
@@ -12872,7 +12872,7 @@
         <v>59830189.120833419</v>
       </c>
     </row>
-    <row r="268" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A268" s="18" t="s">
         <v>102</v>
       </c>
@@ -12917,7 +12917,7 @@
         <v>404502055.98924994</v>
       </c>
     </row>
-    <row r="269" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A269" t="s">
         <v>75</v>
       </c>
@@ -12965,7 +12965,7 @@
         <v>172186685.99542397</v>
       </c>
     </row>
-    <row r="270" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A270" s="22" t="s">
         <v>76</v>
       </c>
@@ -13013,7 +13013,7 @@
         <v>38263707.998983108</v>
       </c>
     </row>
-    <row r="271" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="271" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A271" t="s">
         <v>77</v>
       </c>
@@ -13061,7 +13061,7 @@
         <v>71061171.998111486</v>
       </c>
     </row>
-    <row r="272" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="272" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A272" t="s">
         <v>80</v>
       </c>
@@ -13109,7 +13109,7 @@
         <v>68328049.998184115</v>
       </c>
     </row>
-    <row r="273" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="273" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A273" t="s">
         <v>83</v>
       </c>
@@ -13157,7 +13157,7 @@
         <v>10932487.999709459</v>
       </c>
     </row>
-    <row r="274" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="274" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A274" t="s">
         <v>87</v>
       </c>
@@ -13205,7 +13205,7 @@
         <v>8199365.9997820929</v>
       </c>
     </row>
-    <row r="275" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="275" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A275" t="s">
         <v>88</v>
       </c>
@@ -13253,7 +13253,7 @@
         <v>27331219.999273647</v>
       </c>
     </row>
-    <row r="276" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="276" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A276" t="s">
         <v>89</v>
       </c>
@@ -13301,7 +13301,7 @@
         <v>8199365.9997820929</v>
       </c>
     </row>
-    <row r="277" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A277" s="18" t="s">
         <v>103</v>
       </c>
@@ -13346,7 +13346,7 @@
         <v>31534690.498127222</v>
       </c>
     </row>
-    <row r="278" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="278" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A278" t="s">
         <v>77</v>
       </c>
@@ -13394,7 +13394,7 @@
         <v>24845513.725797206</v>
       </c>
     </row>
-    <row r="279" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="279" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A279" s="2" t="s">
         <v>79</v>
       </c>
@@ -13442,7 +13442,7 @@
         <v>5733580.0905685853</v>
       </c>
     </row>
-    <row r="280" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="280" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A280" s="2" t="s">
         <v>90</v>
       </c>
@@ -13490,7 +13490,7 @@
         <v>955596.68176143093</v>
       </c>
     </row>
-    <row r="281" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="281" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A281" s="28" t="s">
         <v>154</v>
       </c>
@@ -13533,7 +13533,7 @@
         <v>955596.68176143104</v>
       </c>
     </row>
-    <row r="282" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A282" s="18" t="s">
         <v>104</v>
       </c>
@@ -13578,7 +13578,7 @@
         <v>71451386.809868425</v>
       </c>
     </row>
-    <row r="283" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="283" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A283" t="s">
         <v>75</v>
       </c>
@@ -13626,7 +13626,7 @@
         <v>63400526.324249454</v>
       </c>
     </row>
-    <row r="284" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="284" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A284" s="2" t="s">
         <v>82</v>
       </c>
@@ -13674,7 +13674,7 @@
         <v>8050860.485618975</v>
       </c>
     </row>
-    <row r="285" spans="1:12" s="19" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:12" s="19" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A285" s="18" t="s">
         <v>105</v>
       </c>
@@ -13719,7 +13719,7 @@
         <v>3954.38333881579</v>
       </c>
     </row>
-    <row r="286" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="286" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A286" t="s">
         <v>75</v>
       </c>
@@ -13767,7 +13767,7 @@
         <v>2737.650003795547</v>
       </c>
     </row>
-    <row r="287" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="287" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A287" t="s">
         <v>80</v>
       </c>
@@ -13815,7 +13815,7 @@
         <v>1086.3690491252169</v>
       </c>
     </row>
-    <row r="288" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="288" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A288" s="2" t="s">
         <v>91</v>
       </c>
@@ -13863,7 +13863,7 @@
         <v>130.36428589502603</v>
       </c>
     </row>
-    <row r="289" spans="1:12" s="30" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:12" s="30" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A289" s="29" t="s">
         <v>62</v>
       </c>
@@ -13908,7 +13908,7 @@
         <v>190622554.0397763</v>
       </c>
     </row>
-    <row r="290" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="290" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A290" s="2" t="s">
         <v>75</v>
       </c>
@@ -13956,7 +13956,7 @@
         <v>121305261.66167584</v>
       </c>
     </row>
-    <row r="291" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="291" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A291" s="2" t="s">
         <v>88</v>
       </c>
@@ -14004,7 +14004,7 @@
         <v>13932545.477990292</v>
       </c>
     </row>
-    <row r="292" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="292" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A292" s="2" t="s">
         <v>77</v>
       </c>
@@ -14052,7 +14052,7 @@
         <v>50062488.939739235</v>
       </c>
     </row>
-    <row r="293" spans="1:12" s="30" customFormat="1" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:12" s="30" customFormat="1" ht="15.75" hidden="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A293" s="29" t="s">
         <v>155</v>
       </c>
@@ -14097,7 +14097,7 @@
         <v>242257676.2505697</v>
       </c>
     </row>
-    <row r="294" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="294" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A294" s="2" t="s">
         <v>75</v>
       </c>
@@ -14145,7 +14145,7 @@
         <v>165893843.51941183</v>
       </c>
     </row>
-    <row r="295" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="295" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A295" s="2" t="s">
         <v>156</v>
       </c>
@@ -14193,7 +14193,7 @@
         <v>7899706.834257707</v>
       </c>
     </row>
-    <row r="296" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="296" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A296" s="2" t="s">
         <v>77</v>
       </c>
@@ -14241,7 +14241,7 @@
         <v>68464125.896900132</v>
       </c>
     </row>
-    <row r="301" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="301" spans="1:12" x14ac:dyDescent="0.25">
       <c r="H301" s="16"/>
       <c r="I301" s="16"/>
       <c r="J301" s="16"/>
@@ -14340,15 +14340,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{55228539-2602-4D9E-BF99-AB1A3FA50A1F}">
   <dimension ref="A1:W63"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="39.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="11" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="23" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="39.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="11" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="23" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>120</v>
       </c>
@@ -14383,7 +14383,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>123</v>
       </c>
@@ -14418,7 +14418,7 @@
         <v>19943396.373611137</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>140</v>
       </c>
@@ -14486,7 +14486,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>140</v>
       </c>
@@ -14554,7 +14554,7 @@
         <v>19943396.373611137</v>
       </c>
     </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>140</v>
       </c>
@@ -14622,7 +14622,7 @@
         <v>25370340.849170271</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>141</v>
       </c>
@@ -14690,7 +14690,7 @@
         <v>8199365.9997820929</v>
       </c>
     </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>142</v>
       </c>
@@ -14758,7 +14758,7 @@
         <v>41263765.477263942</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>142</v>
       </c>
@@ -14826,7 +14826,7 @@
         <v>13295597.582407426</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>143</v>
       </c>
@@ -14894,7 +14894,7 @@
         <v>158370575.61266673</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>144</v>
       </c>
@@ -14962,7 +14962,7 @@
         <v>130.36428589502603</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>144</v>
       </c>
@@ -15030,7 +15030,7 @@
         <v>217845404.09308761</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>144</v>
       </c>
@@ -15098,7 +15098,7 @@
         <v>8199365.9997820929</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>145</v>
       </c>
@@ -15166,7 +15166,7 @@
         <v>955596.68176143104</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>116</v>
       </c>
@@ -15234,7 +15234,7 @@
         <v>82304159.225267321</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>116</v>
       </c>
@@ -15302,7 +15302,7 @@
         <v>5733580.0905685853</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>116</v>
       </c>
@@ -15370,7 +15370,7 @@
         <v>21467942.204718776</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>116</v>
       </c>
@@ -15438,7 +15438,7 @@
         <v>7899706.834257707</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>116</v>
       </c>
@@ -15506,7 +15506,7 @@
         <v>123285374.16737279</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>146</v>
       </c>
@@ -15574,7 +15574,7 @@
         <v>128159325.48806667</v>
       </c>
     </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="28" t="s">
         <v>154</v>
       </c>
@@ -15642,7 +15642,7 @@
         <v>1169589562.8925073</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>147</v>
       </c>
@@ -15710,7 +15710,7 @@
         <v>955596.68176143093</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>147</v>
       </c>
@@ -15778,7 +15778,7 @@
         <v>2032838786.6183393</v>
       </c>
     </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>147</v>
       </c>
@@ -15813,7 +15813,7 @@
         <v>8050860.485618975</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>148</v>
       </c>
@@ -15848,7 +15848,7 @@
         <v>5733580.0905685853</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>149</v>
       </c>
@@ -15916,7 +15916,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="26" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>149</v>
       </c>
@@ -15984,7 +15984,7 @@
         <v>19943396.373611137</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>156</v>
       </c>
@@ -16052,7 +16052,7 @@
         <v>25370340.849170271</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A28" s="22" t="s">
         <v>150</v>
       </c>
@@ -16120,7 +16120,7 @@
         <v>8199365.9997820929</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A29" s="22" t="s">
         <v>150</v>
       </c>
@@ -16188,7 +16188,7 @@
         <v>41263765.477263942</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A30" s="22" t="s">
         <v>150</v>
       </c>
@@ -16256,7 +16256,7 @@
         <v>13295597.582407426</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A31" s="22" t="s">
         <v>150</v>
       </c>
@@ -16324,7 +16324,7 @@
         <v>158370575.61266673</v>
       </c>
     </row>
-    <row r="32" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A32" s="22" t="s">
         <v>150</v>
       </c>
@@ -16392,7 +16392,7 @@
         <v>130.36428589502603</v>
       </c>
     </row>
-    <row r="33" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A33" s="22" t="s">
         <v>150</v>
       </c>
@@ -16460,7 +16460,7 @@
         <v>217845404.09308761</v>
       </c>
     </row>
-    <row r="34" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>151</v>
       </c>
@@ -16528,7 +16528,7 @@
         <v>8199365.9997820929</v>
       </c>
     </row>
-    <row r="35" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>151</v>
       </c>
@@ -16596,7 +16596,7 @@
         <v>955596.68176143104</v>
       </c>
     </row>
-    <row r="36" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>151</v>
       </c>
@@ -16664,7 +16664,7 @@
         <v>82304159.225267321</v>
       </c>
     </row>
-    <row r="37" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
         <v>152</v>
       </c>
@@ -16732,7 +16732,7 @@
         <v>5733580.0905685853</v>
       </c>
     </row>
-    <row r="38" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>152</v>
       </c>
@@ -16800,7 +16800,7 @@
         <v>21467942.204718776</v>
       </c>
     </row>
-    <row r="39" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>152</v>
       </c>
@@ -16868,7 +16868,7 @@
         <v>7899706.834257707</v>
       </c>
     </row>
-    <row r="40" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
         <v>152</v>
       </c>
@@ -16936,7 +16936,7 @@
         <v>123285374.16737279</v>
       </c>
     </row>
-    <row r="41" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
         <v>152</v>
       </c>
@@ -17004,7 +17004,7 @@
         <v>128159325.48806667</v>
       </c>
     </row>
-    <row r="42" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
         <v>152</v>
       </c>
@@ -17072,7 +17072,7 @@
         <v>1169589562.8925073</v>
       </c>
     </row>
-    <row r="43" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
         <v>152</v>
       </c>
@@ -17140,7 +17140,7 @@
         <v>955596.68176143093</v>
       </c>
     </row>
-    <row r="44" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>152</v>
       </c>
@@ -17208,7 +17208,7 @@
         <v>2032838786.6183393</v>
       </c>
     </row>
-    <row r="45" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
         <v>152</v>
       </c>
@@ -17273,7 +17273,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A46" s="2" t="s">
         <v>152</v>
       </c>
@@ -17351,7 +17351,7 @@
         <v>19900000</v>
       </c>
     </row>
-    <row r="47" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
         <v>152</v>
       </c>
@@ -17429,7 +17429,7 @@
         <v>25400000</v>
       </c>
     </row>
-    <row r="48" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
         <v>152</v>
       </c>
@@ -17507,7 +17507,7 @@
         <v>8200000</v>
       </c>
     </row>
-    <row r="49" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
         <v>152</v>
       </c>
@@ -17585,7 +17585,7 @@
         <v>41300000</v>
       </c>
     </row>
-    <row r="50" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
         <v>152</v>
       </c>
@@ -17663,7 +17663,7 @@
         <v>13300000</v>
       </c>
     </row>
-    <row r="51" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
         <v>153</v>
       </c>
@@ -17741,7 +17741,7 @@
         <v>158400000</v>
       </c>
     </row>
-    <row r="52" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M52" t="s">
         <v>145</v>
       </c>
@@ -17786,7 +17786,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M53" t="s">
         <v>116</v>
       </c>
@@ -17831,7 +17831,7 @@
         <v>217800000</v>
       </c>
     </row>
-    <row r="54" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M54" t="s">
         <v>146</v>
       </c>
@@ -17876,7 +17876,7 @@
         <v>8200000</v>
       </c>
     </row>
-    <row r="55" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M55" t="s">
         <v>154</v>
       </c>
@@ -17921,7 +17921,7 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="56" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M56" t="s">
         <v>147</v>
       </c>
@@ -17966,7 +17966,7 @@
         <v>82300000</v>
       </c>
     </row>
-    <row r="57" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M57" t="s">
         <v>148</v>
       </c>
@@ -18011,7 +18011,7 @@
         <v>5700000</v>
       </c>
     </row>
-    <row r="58" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M58" t="s">
         <v>149</v>
       </c>
@@ -18056,7 +18056,7 @@
         <v>21500000</v>
       </c>
     </row>
-    <row r="59" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M59" t="s">
         <v>156</v>
       </c>
@@ -18101,7 +18101,7 @@
         <v>7900000</v>
       </c>
     </row>
-    <row r="60" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M60" t="s">
         <v>150</v>
       </c>
@@ -18146,7 +18146,7 @@
         <v>123300000</v>
       </c>
     </row>
-    <row r="61" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M61" t="s">
         <v>151</v>
       </c>
@@ -18191,7 +18191,7 @@
         <v>128200000</v>
       </c>
     </row>
-    <row r="62" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M62" t="s">
         <v>152</v>
       </c>
@@ -18236,7 +18236,7 @@
         <v>1169600000</v>
       </c>
     </row>
-    <row r="63" spans="1:23" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:23" x14ac:dyDescent="0.25">
       <c r="M63" t="s">
         <v>153</v>
       </c>
@@ -18290,13 +18290,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{770C77AF-CB50-4854-8654-5465FF2CEF2B}">
   <dimension ref="B2:T19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="39.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B2" s="26" t="s">
         <v>84</v>
       </c>
@@ -18352,7 +18352,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="3" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B3" s="26" t="s">
         <v>81</v>
       </c>
@@ -18424,7 +18424,7 @@
         <v>"Xiamen_Innovax",</v>
       </c>
     </row>
-    <row r="4" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B4" s="26" t="s">
         <v>87</v>
       </c>
@@ -18436,7 +18436,7 @@
         <v>"AJ_Vaccines","BB_NCIPD","Beijing_Institute","Bharat_Biotech","Bilthoven","Biological_E","Centro_de","GSK","Haffkine_Bio","LG_Chem","Merck_Sharp","Panacea_Biotec","PT_Bio","Sanofi_Pasteur","Serum_Institute","Xiamen_Innovax",</v>
       </c>
     </row>
-    <row r="5" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B5" s="26" t="s">
         <v>88</v>
       </c>
@@ -18444,7 +18444,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="6" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B6" s="26" t="s">
         <v>85</v>
       </c>
@@ -18452,7 +18452,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B7" s="26" t="s">
         <v>119</v>
       </c>
@@ -18460,7 +18460,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="8" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B8" s="26" t="s">
         <v>91</v>
       </c>
@@ -18468,7 +18468,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="9" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B9" s="26" t="s">
         <v>77</v>
       </c>
@@ -18476,7 +18476,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="10" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B10" s="26" t="s">
         <v>89</v>
       </c>
@@ -18484,7 +18484,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="11" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B11" s="26" t="s">
         <v>82</v>
       </c>
@@ -18492,7 +18492,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="12" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B12" s="26" t="s">
         <v>79</v>
       </c>
@@ -18500,7 +18500,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="13" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B13" s="26" t="s">
         <v>83</v>
       </c>
@@ -18508,7 +18508,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="14" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B14" s="26" t="s">
         <v>118</v>
       </c>
@@ -18516,7 +18516,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="15" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B15" s="26" t="s">
         <v>80</v>
       </c>
@@ -18524,7 +18524,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="16" spans="2:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:20" x14ac:dyDescent="0.25">
       <c r="B16" s="26" t="s">
         <v>75</v>
       </c>
@@ -18532,7 +18532,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" s="26" t="s">
         <v>90</v>
       </c>
@@ -18540,7 +18540,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="26" t="s">
         <v>156</v>
       </c>
@@ -18548,7 +18548,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" s="26" t="s">
         <v>154</v>
       </c>
@@ -18565,13 +18565,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DF17EB8-02F1-485E-9D81-51CF2F0BE0EA}">
   <dimension ref="A1:K44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="11" width="12" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B1" s="36">
         <v>1</v>
       </c>
@@ -18603,7 +18606,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>123</v>
       </c>
@@ -18638,7 +18641,7 @@
         <v>19900000</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>140</v>
       </c>
@@ -18673,7 +18676,7 @@
         <v>25400000</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>141</v>
       </c>
@@ -18708,7 +18711,7 @@
         <v>8200000</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>142</v>
       </c>
@@ -18743,7 +18746,7 @@
         <v>41300000</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>143</v>
       </c>
@@ -18778,7 +18781,7 @@
         <v>13300000</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>144</v>
       </c>
@@ -18813,7 +18816,7 @@
         <v>158400000</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>145</v>
       </c>
@@ -18848,7 +18851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>116</v>
       </c>
@@ -18883,7 +18886,7 @@
         <v>217800000</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>146</v>
       </c>
@@ -18918,77 +18921,87 @@
         <v>8200000</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>147</v>
       </c>
-      <c r="B11" s="37">
-        <v>60600000</v>
-      </c>
-      <c r="C11" s="37">
-        <v>74600000</v>
-      </c>
-      <c r="D11" s="37">
-        <v>83000000</v>
-      </c>
-      <c r="E11" s="37">
-        <v>81300000</v>
-      </c>
-      <c r="F11" s="37">
-        <v>81100000</v>
-      </c>
-      <c r="G11" s="37">
-        <v>79800000</v>
-      </c>
-      <c r="H11" s="37">
-        <v>81100000</v>
-      </c>
-      <c r="I11" s="37">
-        <v>79900000</v>
-      </c>
-      <c r="J11" s="37">
-        <v>81200000</v>
-      </c>
-      <c r="K11" s="37">
-        <v>82300000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="B11" s="25">
+        <f>B20*17</f>
+        <v>1030200000</v>
+      </c>
+      <c r="C11" s="25">
+        <f t="shared" ref="C11:K11" si="0">C20*17</f>
+        <v>1268200000</v>
+      </c>
+      <c r="D11" s="25">
+        <f t="shared" si="0"/>
+        <v>1411000000</v>
+      </c>
+      <c r="E11" s="25">
+        <f t="shared" si="0"/>
+        <v>1382100000</v>
+      </c>
+      <c r="F11" s="25">
+        <f t="shared" si="0"/>
+        <v>1378700000</v>
+      </c>
+      <c r="G11" s="25">
+        <f t="shared" si="0"/>
+        <v>1356600000</v>
+      </c>
+      <c r="H11" s="25">
+        <f t="shared" si="0"/>
+        <v>1378700000</v>
+      </c>
+      <c r="I11" s="25">
+        <f t="shared" si="0"/>
+        <v>1358300000</v>
+      </c>
+      <c r="J11" s="25">
+        <f t="shared" si="0"/>
+        <v>1380400000</v>
+      </c>
+      <c r="K11" s="25">
+        <f t="shared" si="0"/>
+        <v>1399100000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>148</v>
       </c>
       <c r="B12" s="37">
-        <v>3100000</v>
+        <v>248000000</v>
       </c>
       <c r="C12" s="37">
-        <v>3100000</v>
+        <v>248000000</v>
       </c>
       <c r="D12" s="37">
-        <v>4500000</v>
+        <v>360000000</v>
       </c>
       <c r="E12" s="37">
-        <v>11900000</v>
+        <v>952000000</v>
       </c>
       <c r="F12" s="37">
-        <v>15200000</v>
+        <v>1216000000</v>
       </c>
       <c r="G12" s="37">
-        <v>10600000</v>
+        <v>848000000</v>
       </c>
       <c r="H12" s="37">
-        <v>6900000</v>
+        <v>552000000</v>
       </c>
       <c r="I12" s="37">
-        <v>6900000</v>
+        <v>552000000</v>
       </c>
       <c r="J12" s="37">
-        <v>5500000</v>
+        <v>440000000</v>
       </c>
       <c r="K12" s="37">
-        <v>5700000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+        <v>456000000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>149</v>
       </c>
@@ -19023,7 +19036,7 @@
         <v>21500000</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>150</v>
       </c>
@@ -19058,7 +19071,7 @@
         <v>123300000</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>151</v>
       </c>
@@ -19093,7 +19106,7 @@
         <v>128200000</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>152</v>
       </c>
@@ -19128,7 +19141,7 @@
         <v>1169600000</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>153</v>
       </c>
@@ -19163,7 +19176,7 @@
         <v>1000000</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>156</v>
       </c>
@@ -19198,19 +19211,51 @@
         <v>7900000</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="25"/>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="25"/>
+      <c r="H19" s="25"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="25"/>
+      <c r="K19" s="25"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="B20" s="37">
+        <v>60600000</v>
+      </c>
+      <c r="C20" s="37">
+        <v>74600000</v>
+      </c>
+      <c r="D20" s="37">
+        <v>83000000</v>
+      </c>
+      <c r="E20" s="37">
+        <v>81300000</v>
+      </c>
+      <c r="F20" s="37">
+        <v>81100000</v>
+      </c>
+      <c r="G20" s="37">
+        <v>79800000</v>
+      </c>
+      <c r="H20" s="37">
+        <v>81100000</v>
+      </c>
+      <c r="I20" s="37">
+        <v>79900000</v>
+      </c>
+      <c r="J20" s="37">
+        <v>81200000</v>
+      </c>
+      <c r="K20" s="37">
+        <v>82300000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B21" s="25"/>
       <c r="C21" s="25"/>
       <c r="D21" s="25"/>
@@ -19222,7 +19267,7 @@
       <c r="J21" s="25"/>
       <c r="K21" s="25"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B22" s="25"/>
       <c r="C22" s="25"/>
       <c r="D22" s="25"/>
@@ -19234,7 +19279,7 @@
       <c r="J22" s="25"/>
       <c r="K22" s="25"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B23" s="25"/>
       <c r="C23" s="25"/>
       <c r="D23" s="25"/>
@@ -19246,7 +19291,7 @@
       <c r="J23" s="25"/>
       <c r="K23" s="25"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B24" s="25"/>
       <c r="C24" s="25"/>
       <c r="D24" s="25"/>
@@ -19258,7 +19303,7 @@
       <c r="J24" s="25"/>
       <c r="K24" s="25"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
       <c r="D25" s="25"/>
@@ -19270,7 +19315,7 @@
       <c r="J25" s="25"/>
       <c r="K25" s="25"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B26" s="25"/>
       <c r="C26" s="25"/>
       <c r="D26" s="25"/>
@@ -19282,7 +19327,7 @@
       <c r="J26" s="25"/>
       <c r="K26" s="25"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B27" s="25"/>
       <c r="C27" s="25"/>
       <c r="D27" s="25"/>
@@ -19294,7 +19339,7 @@
       <c r="J27" s="25"/>
       <c r="K27" s="25"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B28" s="25"/>
       <c r="C28" s="25"/>
       <c r="D28" s="25"/>
@@ -19306,7 +19351,7 @@
       <c r="J28" s="25"/>
       <c r="K28" s="25"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B29" s="25"/>
       <c r="C29" s="25"/>
       <c r="D29" s="25"/>
@@ -19318,7 +19363,7 @@
       <c r="J29" s="25"/>
       <c r="K29" s="25"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B30" s="25"/>
       <c r="C30" s="25"/>
       <c r="D30" s="25"/>
@@ -19330,7 +19375,7 @@
       <c r="J30" s="25"/>
       <c r="K30" s="25"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B31" s="25"/>
       <c r="C31" s="25"/>
       <c r="D31" s="25"/>
@@ -19342,7 +19387,7 @@
       <c r="J31" s="25"/>
       <c r="K31" s="25"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B32" s="25"/>
       <c r="C32" s="25"/>
       <c r="D32" s="25"/>
@@ -19354,7 +19399,7 @@
       <c r="J32" s="25"/>
       <c r="K32" s="25"/>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B33" s="25"/>
       <c r="C33" s="25"/>
       <c r="D33" s="25"/>
@@ -19366,7 +19411,7 @@
       <c r="J33" s="25"/>
       <c r="K33" s="25"/>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B34" s="25"/>
       <c r="C34" s="25"/>
       <c r="D34" s="25"/>
@@ -19378,7 +19423,7 @@
       <c r="J34" s="25"/>
       <c r="K34" s="25"/>
     </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B35" s="25"/>
       <c r="C35" s="25"/>
       <c r="D35" s="25"/>
@@ -19390,7 +19435,7 @@
       <c r="J35" s="25"/>
       <c r="K35" s="25"/>
     </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B36" s="25"/>
       <c r="C36" s="25"/>
       <c r="D36" s="25"/>
@@ -19402,7 +19447,7 @@
       <c r="J36" s="25"/>
       <c r="K36" s="25"/>
     </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B37" s="25"/>
       <c r="C37" s="25"/>
       <c r="D37" s="25"/>
@@ -19414,7 +19459,7 @@
       <c r="J37" s="25"/>
       <c r="K37" s="25"/>
     </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B38" s="25"/>
       <c r="C38" s="25"/>
       <c r="D38" s="25"/>
@@ -19426,7 +19471,7 @@
       <c r="J38" s="25"/>
       <c r="K38" s="25"/>
     </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B39" s="25"/>
       <c r="C39" s="25"/>
       <c r="D39" s="25"/>
@@ -19438,7 +19483,7 @@
       <c r="J39" s="25"/>
       <c r="K39" s="25"/>
     </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B40" s="25"/>
       <c r="C40" s="25"/>
       <c r="D40" s="25"/>
@@ -19450,7 +19495,7 @@
       <c r="J40" s="25"/>
       <c r="K40" s="25"/>
     </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B41" s="25"/>
       <c r="C41" s="25"/>
       <c r="D41" s="25"/>
@@ -19462,7 +19507,7 @@
       <c r="J41" s="25"/>
       <c r="K41" s="25"/>
     </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B42" s="25"/>
       <c r="C42" s="25"/>
       <c r="D42" s="25"/>
@@ -19474,7 +19519,7 @@
       <c r="J42" s="25"/>
       <c r="K42" s="25"/>
     </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B43" s="25"/>
       <c r="C43" s="25"/>
       <c r="D43" s="25"/>
@@ -19486,7 +19531,7 @@
       <c r="J43" s="25"/>
       <c r="K43" s="25"/>
     </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B44" s="25"/>
       <c r="C44" s="25"/>
       <c r="D44" s="25"/>

</xml_diff>

<commit_message>
updated prod cap to work; working starting tenders for model
</commit_message>
<xml_diff>
--- a/production_capacity_updated.xlsx
+++ b/production_capacity_updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="13_ncr:1_{391AB4AD-8E06-448B-8305-29E04006C88F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{318C915B-7EBB-4C2E-AB54-76CE7BB3ECDA}"/>
+  <xr:revisionPtr revIDLastSave="92" documentId="13_ncr:1_{391AB4AD-8E06-448B-8305-29E04006C88F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F77F21EE-8157-4E23-95E5-4D730731A823}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="4" xr2:uid="{752E71BE-3FD4-4CCA-ABF0-6C5710D300B4}"/>
   </bookViews>
@@ -29,7 +29,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId6"/>
+    <pivotCache cacheId="3" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -710,7 +710,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -783,6 +783,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF098658"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="10">
@@ -937,7 +943,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1009,6 +1015,12 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1798,7 +1810,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B95A2301-B56D-4CF8-964C-AEC6E5E61117}" name="PivotTable3" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{B95A2301-B56D-4CF8-964C-AEC6E5E61117}" name="PivotTable3" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="M3:W22" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField axis="axisRow" showAll="0">
@@ -3666,7 +3678,7 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="43" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="4" t="s">
@@ -3684,7 +3696,7 @@
       <c r="L2" s="6"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="43" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="4" t="s">
@@ -3722,7 +3734,7 @@
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" s="41" t="s">
+      <c r="A4" s="43" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -3760,7 +3772,7 @@
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="43" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="4" t="s">
@@ -3798,7 +3810,7 @@
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" s="41" t="s">
+      <c r="A6" s="43" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="4" t="s">
@@ -3836,7 +3848,7 @@
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" s="41" t="s">
+      <c r="A7" s="43" t="s">
         <v>18</v>
       </c>
       <c r="B7" s="4" t="s">
@@ -3866,7 +3878,7 @@
       <c r="L7" s="6"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" s="41" t="s">
+      <c r="A8" s="43" t="s">
         <v>18</v>
       </c>
       <c r="B8" s="4" t="s">
@@ -3896,7 +3908,7 @@
       <c r="L8" s="6"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" s="41" t="s">
+      <c r="A9" s="43" t="s">
         <v>18</v>
       </c>
       <c r="B9" s="4" t="s">
@@ -3926,7 +3938,7 @@
       <c r="L9" s="6"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" s="41" t="s">
+      <c r="A10" s="43" t="s">
         <v>18</v>
       </c>
       <c r="B10" s="4" t="s">
@@ -3956,7 +3968,7 @@
       <c r="L10" s="6"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A11" s="41" t="s">
+      <c r="A11" s="43" t="s">
         <v>19</v>
       </c>
       <c r="B11" s="4" t="s">
@@ -3994,7 +4006,7 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A12" s="41" t="s">
+      <c r="A12" s="43" t="s">
         <v>19</v>
       </c>
       <c r="B12" s="4" t="s">
@@ -4032,7 +4044,7 @@
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A13" s="41" t="s">
+      <c r="A13" s="43" t="s">
         <v>19</v>
       </c>
       <c r="B13" s="4" t="s">
@@ -4070,7 +4082,7 @@
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A14" s="41" t="s">
+      <c r="A14" s="43" t="s">
         <v>19</v>
       </c>
       <c r="B14" s="4" t="s">
@@ -4144,7 +4156,7 @@
       <c r="L16" s="6"/>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A17" s="41" t="s">
+      <c r="A17" s="43" t="s">
         <v>22</v>
       </c>
       <c r="B17" s="4" t="s">
@@ -4162,7 +4174,7 @@
       <c r="L17" s="6"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A18" s="41" t="s">
+      <c r="A18" s="43" t="s">
         <v>22</v>
       </c>
       <c r="B18" s="4" t="s">
@@ -4200,7 +4212,7 @@
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A19" s="41" t="s">
+      <c r="A19" s="43" t="s">
         <v>22</v>
       </c>
       <c r="B19" s="4" t="s">
@@ -4238,7 +4250,7 @@
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A20" s="41" t="s">
+      <c r="A20" s="43" t="s">
         <v>22</v>
       </c>
       <c r="B20" s="4" t="s">
@@ -4276,7 +4288,7 @@
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A21" s="41" t="s">
+      <c r="A21" s="43" t="s">
         <v>22</v>
       </c>
       <c r="B21" s="4" t="s">
@@ -4314,7 +4326,7 @@
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A22" s="41" t="s">
+      <c r="A22" s="43" t="s">
         <v>23</v>
       </c>
       <c r="B22" s="4" t="s">
@@ -4332,7 +4344,7 @@
       <c r="L22" s="6"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A23" s="41" t="s">
+      <c r="A23" s="43" t="s">
         <v>23</v>
       </c>
       <c r="B23" s="4" t="s">
@@ -4370,7 +4382,7 @@
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A24" s="41" t="s">
+      <c r="A24" s="43" t="s">
         <v>23</v>
       </c>
       <c r="B24" s="4" t="s">
@@ -4388,7 +4400,7 @@
       <c r="L24" s="6"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A25" s="41" t="s">
+      <c r="A25" s="43" t="s">
         <v>23</v>
       </c>
       <c r="B25" s="4" t="s">
@@ -4418,7 +4430,7 @@
       <c r="L25" s="6"/>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A26" s="41" t="s">
+      <c r="A26" s="43" t="s">
         <v>23</v>
       </c>
       <c r="B26" s="4" t="s">
@@ -4474,7 +4486,7 @@
       <c r="L27" s="6"/>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A28" s="41" t="s">
+      <c r="A28" s="43" t="s">
         <v>25</v>
       </c>
       <c r="B28" s="4" t="s">
@@ -4512,7 +4524,7 @@
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A29" s="41" t="s">
+      <c r="A29" s="43" t="s">
         <v>25</v>
       </c>
       <c r="B29" s="4" t="s">
@@ -4542,7 +4554,7 @@
       <c r="L29" s="6"/>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A30" s="41" t="s">
+      <c r="A30" s="43" t="s">
         <v>25</v>
       </c>
       <c r="B30" s="4" t="s">
@@ -4568,7 +4580,7 @@
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A31" s="41" t="s">
+      <c r="A31" s="43" t="s">
         <v>26</v>
       </c>
       <c r="B31" s="4" t="s">
@@ -4606,7 +4618,7 @@
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A32" s="41" t="s">
+      <c r="A32" s="43" t="s">
         <v>26</v>
       </c>
       <c r="B32" s="4" t="s">
@@ -4632,7 +4644,7 @@
       <c r="L32" s="6"/>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A33" s="41" t="s">
+      <c r="A33" s="43" t="s">
         <v>26</v>
       </c>
       <c r="B33" s="4" t="s">
@@ -4670,7 +4682,7 @@
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A34" s="41" t="s">
+      <c r="A34" s="43" t="s">
         <v>27</v>
       </c>
       <c r="B34" s="4" t="s">
@@ -4708,7 +4720,7 @@
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A35" s="41" t="s">
+      <c r="A35" s="43" t="s">
         <v>27</v>
       </c>
       <c r="B35" s="4" t="s">
@@ -4738,7 +4750,7 @@
       <c r="L35" s="6"/>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A36" s="41" t="s">
+      <c r="A36" s="43" t="s">
         <v>27</v>
       </c>
       <c r="B36" s="4" t="s">
@@ -4764,7 +4776,7 @@
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A37" s="41" t="s">
+      <c r="A37" s="43" t="s">
         <v>28</v>
       </c>
       <c r="B37" s="4" t="s">
@@ -4802,7 +4814,7 @@
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A38" s="41" t="s">
+      <c r="A38" s="43" t="s">
         <v>28</v>
       </c>
       <c r="B38" s="4" t="s">
@@ -4828,7 +4840,7 @@
       <c r="L38" s="6"/>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A39" s="41" t="s">
+      <c r="A39" s="43" t="s">
         <v>29</v>
       </c>
       <c r="B39" s="4" t="s">
@@ -4866,7 +4878,7 @@
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A40" s="41" t="s">
+      <c r="A40" s="43" t="s">
         <v>29</v>
       </c>
       <c r="B40" s="4" t="s">
@@ -4892,7 +4904,7 @@
       <c r="L40" s="6"/>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A41" s="41" t="s">
+      <c r="A41" s="43" t="s">
         <v>29</v>
       </c>
       <c r="B41" s="4" t="s">
@@ -4930,7 +4942,7 @@
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A42" s="41" t="s">
+      <c r="A42" s="43" t="s">
         <v>30</v>
       </c>
       <c r="B42" s="4" t="s">
@@ -4968,7 +4980,7 @@
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A43" s="41" t="s">
+      <c r="A43" s="43" t="s">
         <v>30</v>
       </c>
       <c r="B43" s="4" t="s">
@@ -4986,7 +4998,7 @@
       <c r="L43" s="6"/>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A44" s="41" t="s">
+      <c r="A44" s="43" t="s">
         <v>30</v>
       </c>
       <c r="B44" s="4" t="s">
@@ -5024,7 +5036,7 @@
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A45" s="41" t="s">
+      <c r="A45" s="43" t="s">
         <v>31</v>
       </c>
       <c r="B45" s="4" t="s">
@@ -5042,7 +5054,7 @@
       <c r="L45" s="6"/>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A46" s="41" t="s">
+      <c r="A46" s="43" t="s">
         <v>31</v>
       </c>
       <c r="B46" s="4" t="s">
@@ -5080,7 +5092,7 @@
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A47" s="41" t="s">
+      <c r="A47" s="43" t="s">
         <v>31</v>
       </c>
       <c r="B47" s="4" t="s">
@@ -5118,7 +5130,7 @@
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A48" s="41" t="s">
+      <c r="A48" s="43" t="s">
         <v>31</v>
       </c>
       <c r="B48" s="4" t="s">
@@ -5156,7 +5168,7 @@
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A49" s="41" t="s">
+      <c r="A49" s="43" t="s">
         <v>31</v>
       </c>
       <c r="B49" s="4" t="s">
@@ -5194,7 +5206,7 @@
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A50" s="41" t="s">
+      <c r="A50" s="43" t="s">
         <v>32</v>
       </c>
       <c r="B50" s="4" t="s">
@@ -5212,7 +5224,7 @@
       <c r="L50" s="6"/>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A51" s="41" t="s">
+      <c r="A51" s="43" t="s">
         <v>32</v>
       </c>
       <c r="B51" s="4" t="s">
@@ -5230,7 +5242,7 @@
       <c r="L51" s="6"/>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A52" s="41" t="s">
+      <c r="A52" s="43" t="s">
         <v>32</v>
       </c>
       <c r="B52" s="4" t="s">
@@ -5248,7 +5260,7 @@
       <c r="L52" s="6"/>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A53" s="41" t="s">
+      <c r="A53" s="43" t="s">
         <v>32</v>
       </c>
       <c r="B53" s="4" t="s">
@@ -5286,7 +5298,7 @@
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A54" s="41" t="s">
+      <c r="A54" s="43" t="s">
         <v>33</v>
       </c>
       <c r="B54" s="4" t="s">
@@ -5324,7 +5336,7 @@
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A55" s="41" t="s">
+      <c r="A55" s="43" t="s">
         <v>33</v>
       </c>
       <c r="B55" s="4" t="s">
@@ -5362,7 +5374,7 @@
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A56" s="41" t="s">
+      <c r="A56" s="43" t="s">
         <v>33</v>
       </c>
       <c r="B56" s="4" t="s">
@@ -5400,7 +5412,7 @@
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A57" s="41" t="s">
+      <c r="A57" s="43" t="s">
         <v>33</v>
       </c>
       <c r="B57" s="4" t="s">
@@ -5438,7 +5450,7 @@
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A58" s="41" t="s">
+      <c r="A58" s="43" t="s">
         <v>34</v>
       </c>
       <c r="B58" s="4" t="s">
@@ -5476,7 +5488,7 @@
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A59" s="41" t="s">
+      <c r="A59" s="43" t="s">
         <v>34</v>
       </c>
       <c r="B59" s="4" t="s">
@@ -5514,7 +5526,7 @@
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A60" s="41" t="s">
+      <c r="A60" s="43" t="s">
         <v>34</v>
       </c>
       <c r="B60" s="4" t="s">
@@ -5552,7 +5564,7 @@
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A61" s="41" t="s">
+      <c r="A61" s="43" t="s">
         <v>34</v>
       </c>
       <c r="B61" s="4" t="s">
@@ -5572,7 +5584,7 @@
       <c r="L61" s="6"/>
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A62" s="41" t="s">
+      <c r="A62" s="43" t="s">
         <v>35</v>
       </c>
       <c r="B62" s="4" t="s">
@@ -5610,7 +5622,7 @@
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A63" s="41" t="s">
+      <c r="A63" s="43" t="s">
         <v>35</v>
       </c>
       <c r="B63" s="4" t="s">
@@ -5648,7 +5660,7 @@
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A64" s="41" t="s">
+      <c r="A64" s="43" t="s">
         <v>35</v>
       </c>
       <c r="B64" s="4" t="s">
@@ -5686,7 +5698,7 @@
       </c>
     </row>
     <row r="65" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A65" s="41" t="s">
+      <c r="A65" s="43" t="s">
         <v>36</v>
       </c>
       <c r="B65" s="4" t="s">
@@ -5704,7 +5716,7 @@
       <c r="L65" s="6"/>
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A66" s="41" t="s">
+      <c r="A66" s="43" t="s">
         <v>36</v>
       </c>
       <c r="B66" s="4" t="s">
@@ -5742,7 +5754,7 @@
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A67" s="41" t="s">
+      <c r="A67" s="43" t="s">
         <v>36</v>
       </c>
       <c r="B67" s="4" t="s">
@@ -5780,7 +5792,7 @@
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A68" s="41" t="s">
+      <c r="A68" s="43" t="s">
         <v>36</v>
       </c>
       <c r="B68" s="4" t="s">
@@ -5818,7 +5830,7 @@
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A69" s="41" t="s">
+      <c r="A69" s="43" t="s">
         <v>36</v>
       </c>
       <c r="B69" s="4" t="s">
@@ -5856,7 +5868,7 @@
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A70" s="41" t="s">
+      <c r="A70" s="43" t="s">
         <v>37</v>
       </c>
       <c r="B70" s="4" t="s">
@@ -5874,7 +5886,7 @@
       <c r="L70" s="6"/>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A71" s="41" t="s">
+      <c r="A71" s="43" t="s">
         <v>37</v>
       </c>
       <c r="B71" s="4" t="s">
@@ -5912,7 +5924,7 @@
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A72" s="41" t="s">
+      <c r="A72" s="43" t="s">
         <v>37</v>
       </c>
       <c r="B72" s="4" t="s">
@@ -5930,7 +5942,7 @@
       <c r="L72" s="6"/>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A73" s="41" t="s">
+      <c r="A73" s="43" t="s">
         <v>37</v>
       </c>
       <c r="B73" s="4" t="s">
@@ -5960,7 +5972,7 @@
       <c r="L73" s="6"/>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A74" s="41" t="s">
+      <c r="A74" s="43" t="s">
         <v>37</v>
       </c>
       <c r="B74" s="4" t="s">
@@ -5998,7 +6010,7 @@
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A75" s="41" t="s">
+      <c r="A75" s="43" t="s">
         <v>38</v>
       </c>
       <c r="B75" s="4" t="s">
@@ -6028,7 +6040,7 @@
       </c>
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A76" s="41" t="s">
+      <c r="A76" s="43" t="s">
         <v>38</v>
       </c>
       <c r="B76" s="4" t="s">
@@ -6092,7 +6104,7 @@
       </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A78" s="41" t="s">
+      <c r="A78" s="43" t="s">
         <v>40</v>
       </c>
       <c r="B78" s="4" t="s">
@@ -6130,7 +6142,7 @@
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A79" s="41" t="s">
+      <c r="A79" s="43" t="s">
         <v>40</v>
       </c>
       <c r="B79" s="4" t="s">
@@ -6168,7 +6180,7 @@
       </c>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A80" s="41" t="s">
+      <c r="A80" s="43" t="s">
         <v>40</v>
       </c>
       <c r="B80" s="4" t="s">
@@ -6206,7 +6218,7 @@
       </c>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A81" s="41" t="s">
+      <c r="A81" s="43" t="s">
         <v>40</v>
       </c>
       <c r="B81" s="4" t="s">
@@ -6244,7 +6256,7 @@
       </c>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A82" s="41" t="s">
+      <c r="A82" s="43" t="s">
         <v>41</v>
       </c>
       <c r="B82" s="4" t="s">
@@ -6282,7 +6294,7 @@
       </c>
     </row>
     <row r="83" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A83" s="41" t="s">
+      <c r="A83" s="43" t="s">
         <v>41</v>
       </c>
       <c r="B83" s="4" t="s">
@@ -6320,7 +6332,7 @@
       </c>
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A84" s="41" t="s">
+      <c r="A84" s="43" t="s">
         <v>41</v>
       </c>
       <c r="B84" s="4" t="s">
@@ -6358,7 +6370,7 @@
       </c>
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A85" s="41" t="s">
+      <c r="A85" s="43" t="s">
         <v>41</v>
       </c>
       <c r="B85" s="4" t="s">
@@ -6396,7 +6408,7 @@
       </c>
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A86" s="41" t="s">
+      <c r="A86" s="43" t="s">
         <v>42</v>
       </c>
       <c r="B86" s="4" t="s">
@@ -6434,7 +6446,7 @@
       </c>
     </row>
     <row r="87" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A87" s="41" t="s">
+      <c r="A87" s="43" t="s">
         <v>42</v>
       </c>
       <c r="B87" s="4" t="s">
@@ -6452,7 +6464,7 @@
       <c r="L87" s="6"/>
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A88" s="41" t="s">
+      <c r="A88" s="43" t="s">
         <v>42</v>
       </c>
       <c r="B88" s="4" t="s">
@@ -6490,7 +6502,7 @@
       </c>
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A89" s="41" t="s">
+      <c r="A89" s="43" t="s">
         <v>42</v>
       </c>
       <c r="B89" s="4" t="s">
@@ -6528,7 +6540,7 @@
       </c>
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A90" s="42" t="s">
+      <c r="A90" s="44" t="s">
         <v>43</v>
       </c>
       <c r="B90" s="4" t="s">
@@ -6546,7 +6558,7 @@
       <c r="L90" s="6"/>
     </row>
     <row r="91" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A91" s="43" t="s">
+      <c r="A91" s="45" t="s">
         <v>43</v>
       </c>
       <c r="B91" s="4" t="s">
@@ -6584,7 +6596,7 @@
       </c>
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A92" s="43" t="s">
+      <c r="A92" s="45" t="s">
         <v>43</v>
       </c>
       <c r="B92" s="4" t="s">
@@ -6622,7 +6634,7 @@
       </c>
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A93" s="43" t="s">
+      <c r="A93" s="45" t="s">
         <v>43</v>
       </c>
       <c r="B93" s="4" t="s">
@@ -6660,7 +6672,7 @@
       </c>
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A94" s="44" t="s">
+      <c r="A94" s="46" t="s">
         <v>43</v>
       </c>
       <c r="B94" s="4" t="s">
@@ -6698,7 +6710,7 @@
       </c>
     </row>
     <row r="95" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A95" s="41" t="s">
+      <c r="A95" s="43" t="s">
         <v>44</v>
       </c>
       <c r="B95" s="4" t="s">
@@ -6736,7 +6748,7 @@
       </c>
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A96" s="41" t="s">
+      <c r="A96" s="43" t="s">
         <v>44</v>
       </c>
       <c r="B96" s="4" t="s">
@@ -6774,7 +6786,7 @@
       </c>
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A97" s="41" t="s">
+      <c r="A97" s="43" t="s">
         <v>44</v>
       </c>
       <c r="B97" s="4" t="s">
@@ -6812,7 +6824,7 @@
       </c>
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A98" s="41" t="s">
+      <c r="A98" s="43" t="s">
         <v>45</v>
       </c>
       <c r="B98" s="4" t="s">
@@ -6842,7 +6854,7 @@
       </c>
     </row>
     <row r="99" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A99" s="41" t="s">
+      <c r="A99" s="43" t="s">
         <v>45</v>
       </c>
       <c r="B99" s="4" t="s">
@@ -6860,7 +6872,7 @@
       <c r="L99" s="6"/>
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A100" s="41" t="s">
+      <c r="A100" s="43" t="s">
         <v>45</v>
       </c>
       <c r="B100" s="4" t="s">
@@ -6886,7 +6898,7 @@
       <c r="L100" s="6"/>
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A101" s="41" t="s">
+      <c r="A101" s="43" t="s">
         <v>46</v>
       </c>
       <c r="B101" s="4" t="s">
@@ -6924,7 +6936,7 @@
       </c>
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A102" s="41" t="s">
+      <c r="A102" s="43" t="s">
         <v>46</v>
       </c>
       <c r="B102" s="4" t="s">
@@ -6942,7 +6954,7 @@
       <c r="L102" s="6"/>
     </row>
     <row r="103" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A103" s="41" t="s">
+      <c r="A103" s="43" t="s">
         <v>46</v>
       </c>
       <c r="B103" s="4" t="s">
@@ -6968,7 +6980,7 @@
       <c r="L103" s="6"/>
     </row>
     <row r="104" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A104" s="41" t="s">
+      <c r="A104" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B104" s="4" t="s">
@@ -6998,7 +7010,7 @@
       </c>
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A105" s="41" t="s">
+      <c r="A105" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B105" s="4" t="s">
@@ -7026,7 +7038,7 @@
       <c r="L105" s="6"/>
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A106" s="41" t="s">
+      <c r="A106" s="43" t="s">
         <v>47</v>
       </c>
       <c r="B106" s="4" t="s">
@@ -7062,7 +7074,7 @@
       </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A107" s="41" t="s">
+      <c r="A107" s="43" t="s">
         <v>48</v>
       </c>
       <c r="B107" s="4" t="s">
@@ -7100,7 +7112,7 @@
       </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A108" s="41" t="s">
+      <c r="A108" s="43" t="s">
         <v>48</v>
       </c>
       <c r="B108" s="4" t="s">
@@ -7138,7 +7150,7 @@
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A109" s="41" t="s">
+      <c r="A109" s="43" t="s">
         <v>48</v>
       </c>
       <c r="B109" s="4" t="s">
@@ -7156,7 +7168,7 @@
       <c r="L109" s="6"/>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A110" s="41" t="s">
+      <c r="A110" s="43" t="s">
         <v>49</v>
       </c>
       <c r="B110" s="4" t="s">
@@ -7194,7 +7206,7 @@
       </c>
     </row>
     <row r="111" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A111" s="41" t="s">
+      <c r="A111" s="43" t="s">
         <v>49</v>
       </c>
       <c r="B111" s="4" t="s">
@@ -7232,7 +7244,7 @@
       </c>
     </row>
     <row r="112" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A112" s="41" t="s">
+      <c r="A112" s="43" t="s">
         <v>49</v>
       </c>
       <c r="B112" s="4" t="s">
@@ -7268,7 +7280,7 @@
       </c>
     </row>
     <row r="113" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A113" s="41" t="s">
+      <c r="A113" s="43" t="s">
         <v>49</v>
       </c>
       <c r="B113" s="4" t="s">
@@ -7306,7 +7318,7 @@
       </c>
     </row>
     <row r="114" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A114" s="41" t="s">
+      <c r="A114" s="43" t="s">
         <v>50</v>
       </c>
       <c r="B114" s="4" t="s">
@@ -7344,7 +7356,7 @@
       </c>
     </row>
     <row r="115" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A115" s="41" t="s">
+      <c r="A115" s="43" t="s">
         <v>50</v>
       </c>
       <c r="B115" s="4" t="s">
@@ -7382,7 +7394,7 @@
       </c>
     </row>
     <row r="116" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A116" s="41" t="s">
+      <c r="A116" s="43" t="s">
         <v>50</v>
       </c>
       <c r="B116" s="4" t="s">
@@ -7420,7 +7432,7 @@
       </c>
     </row>
     <row r="117" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A117" s="41" t="s">
+      <c r="A117" s="43" t="s">
         <v>50</v>
       </c>
       <c r="B117" s="4" t="s">
@@ -7458,7 +7470,7 @@
       </c>
     </row>
     <row r="118" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A118" s="41" t="s">
+      <c r="A118" s="43" t="s">
         <v>50</v>
       </c>
       <c r="B118" s="4" t="s">
@@ -7532,7 +7544,7 @@
       </c>
     </row>
     <row r="120" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A120" s="41" t="s">
+      <c r="A120" s="43" t="s">
         <v>52</v>
       </c>
       <c r="B120" s="4" t="s">
@@ -7550,7 +7562,7 @@
       <c r="L120" s="6"/>
     </row>
     <row r="121" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A121" s="41" t="s">
+      <c r="A121" s="43" t="s">
         <v>52</v>
       </c>
       <c r="B121" s="4" t="s">
@@ -7582,7 +7594,7 @@
       </c>
     </row>
     <row r="122" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A122" s="41" t="s">
+      <c r="A122" s="43" t="s">
         <v>52</v>
       </c>
       <c r="B122" s="4" t="s">
@@ -7620,7 +7632,7 @@
       </c>
     </row>
     <row r="123" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A123" s="41" t="s">
+      <c r="A123" s="43" t="s">
         <v>53</v>
       </c>
       <c r="B123" s="4" t="s">
@@ -7658,7 +7670,7 @@
       </c>
     </row>
     <row r="124" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A124" s="41" t="s">
+      <c r="A124" s="43" t="s">
         <v>53</v>
       </c>
       <c r="B124" s="4" t="s">
@@ -7696,7 +7708,7 @@
       </c>
     </row>
     <row r="125" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A125" s="41" t="s">
+      <c r="A125" s="43" t="s">
         <v>53</v>
       </c>
       <c r="B125" s="4" t="s">
@@ -7734,7 +7746,7 @@
       </c>
     </row>
     <row r="126" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A126" s="41" t="s">
+      <c r="A126" s="43" t="s">
         <v>54</v>
       </c>
       <c r="B126" s="4" t="s">
@@ -7752,7 +7764,7 @@
       <c r="L126" s="6"/>
     </row>
     <row r="127" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A127" s="41" t="s">
+      <c r="A127" s="43" t="s">
         <v>54</v>
       </c>
       <c r="B127" s="4" t="s">
@@ -7770,7 +7782,7 @@
       <c r="L127" s="6"/>
     </row>
     <row r="128" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A128" s="41" t="s">
+      <c r="A128" s="43" t="s">
         <v>54</v>
       </c>
       <c r="B128" s="4" t="s">
@@ -7788,7 +7800,7 @@
       <c r="L128" s="6"/>
     </row>
     <row r="129" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A129" s="41" t="s">
+      <c r="A129" s="43" t="s">
         <v>54</v>
       </c>
       <c r="B129" s="4" t="s">
@@ -7808,7 +7820,7 @@
       <c r="L129" s="6"/>
     </row>
     <row r="130" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A130" s="41" t="s">
+      <c r="A130" s="43" t="s">
         <v>55</v>
       </c>
       <c r="B130" s="4" t="s">
@@ -7826,7 +7838,7 @@
       <c r="L130" s="6"/>
     </row>
     <row r="131" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A131" s="41" t="s">
+      <c r="A131" s="43" t="s">
         <v>55</v>
       </c>
       <c r="B131" s="4" t="s">
@@ -7864,7 +7876,7 @@
       </c>
     </row>
     <row r="132" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A132" s="41" t="s">
+      <c r="A132" s="43" t="s">
         <v>55</v>
       </c>
       <c r="B132" s="4" t="s">
@@ -7902,7 +7914,7 @@
       </c>
     </row>
     <row r="133" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A133" s="41" t="s">
+      <c r="A133" s="43" t="s">
         <v>55</v>
       </c>
       <c r="B133" s="4" t="s">
@@ -7940,7 +7952,7 @@
       </c>
     </row>
     <row r="134" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A134" s="41" t="s">
+      <c r="A134" s="43" t="s">
         <v>55</v>
       </c>
       <c r="B134" s="4" t="s">
@@ -7978,7 +7990,7 @@
       </c>
     </row>
     <row r="135" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A135" s="41" t="s">
+      <c r="A135" s="43" t="s">
         <v>56</v>
       </c>
       <c r="B135" s="4" t="s">
@@ -8016,7 +8028,7 @@
       </c>
     </row>
     <row r="136" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A136" s="41" t="s">
+      <c r="A136" s="43" t="s">
         <v>56</v>
       </c>
       <c r="B136" s="4" t="s">
@@ -8054,7 +8066,7 @@
       </c>
     </row>
     <row r="137" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A137" s="41" t="s">
+      <c r="A137" s="43" t="s">
         <v>57</v>
       </c>
       <c r="B137" s="4" t="s">
@@ -8092,7 +8104,7 @@
       </c>
     </row>
     <row r="138" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A138" s="41" t="s">
+      <c r="A138" s="43" t="s">
         <v>57</v>
       </c>
       <c r="B138" s="4" t="s">
@@ -8130,7 +8142,7 @@
       </c>
     </row>
     <row r="139" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A139" s="41" t="s">
+      <c r="A139" s="43" t="s">
         <v>57</v>
       </c>
       <c r="B139" s="4" t="s">
@@ -8168,7 +8180,7 @@
       </c>
     </row>
     <row r="140" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A140" s="41" t="s">
+      <c r="A140" s="43" t="s">
         <v>57</v>
       </c>
       <c r="B140" s="4" t="s">
@@ -8244,7 +8256,7 @@
       </c>
     </row>
     <row r="142" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A142" s="41" t="s">
+      <c r="A142" s="43" t="s">
         <v>59</v>
       </c>
       <c r="B142" s="4" t="s">
@@ -8282,7 +8294,7 @@
       </c>
     </row>
     <row r="143" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A143" s="41" t="s">
+      <c r="A143" s="43" t="s">
         <v>59</v>
       </c>
       <c r="B143" s="4" t="s">
@@ -8320,7 +8332,7 @@
       </c>
     </row>
     <row r="144" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A144" s="41" t="s">
+      <c r="A144" s="43" t="s">
         <v>59</v>
       </c>
       <c r="B144" s="4" t="s">
@@ -8358,7 +8370,7 @@
       </c>
     </row>
     <row r="145" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A145" s="41" t="s">
+      <c r="A145" s="43" t="s">
         <v>59</v>
       </c>
       <c r="B145" s="4" t="s">
@@ -8386,7 +8398,7 @@
       </c>
     </row>
     <row r="146" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A146" s="41" t="s">
+      <c r="A146" s="43" t="s">
         <v>60</v>
       </c>
       <c r="B146" s="4" t="s">
@@ -8424,7 +8436,7 @@
       </c>
     </row>
     <row r="147" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A147" s="41" t="s">
+      <c r="A147" s="43" t="s">
         <v>60</v>
       </c>
       <c r="B147" s="4" t="s">
@@ -8462,7 +8474,7 @@
       </c>
     </row>
     <row r="148" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A148" s="41" t="s">
+      <c r="A148" s="43" t="s">
         <v>60</v>
       </c>
       <c r="B148" s="4" t="s">
@@ -8500,7 +8512,7 @@
       </c>
     </row>
     <row r="149" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A149" s="41" t="s">
+      <c r="A149" s="43" t="s">
         <v>60</v>
       </c>
       <c r="B149" s="4" t="s">
@@ -8538,7 +8550,7 @@
       </c>
     </row>
     <row r="150" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A150" s="41" t="s">
+      <c r="A150" s="43" t="s">
         <v>61</v>
       </c>
       <c r="B150" s="4" t="s">
@@ -8576,7 +8588,7 @@
       </c>
     </row>
     <row r="151" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A151" s="41" t="s">
+      <c r="A151" s="43" t="s">
         <v>61</v>
       </c>
       <c r="B151" s="4" t="s">
@@ -8614,7 +8626,7 @@
       </c>
     </row>
     <row r="152" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A152" s="41" t="s">
+      <c r="A152" s="43" t="s">
         <v>61</v>
       </c>
       <c r="B152" s="4" t="s">
@@ -8652,7 +8664,7 @@
       </c>
     </row>
     <row r="153" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A153" s="41" t="s">
+      <c r="A153" s="43" t="s">
         <v>62</v>
       </c>
       <c r="B153" s="4" t="s">
@@ -8690,7 +8702,7 @@
       </c>
     </row>
     <row r="154" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A154" s="41" t="s">
+      <c r="A154" s="43" t="s">
         <v>62</v>
       </c>
       <c r="B154" s="4" t="s">
@@ -8728,7 +8740,7 @@
       </c>
     </row>
     <row r="155" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A155" s="41" t="s">
+      <c r="A155" s="43" t="s">
         <v>62</v>
       </c>
       <c r="B155" s="4" t="s">
@@ -8766,7 +8778,7 @@
       </c>
     </row>
     <row r="156" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A156" s="41" t="s">
+      <c r="A156" s="43" t="s">
         <v>62</v>
       </c>
       <c r="B156" s="4" t="s">
@@ -8804,7 +8816,7 @@
       </c>
     </row>
     <row r="157" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A157" s="41" t="s">
+      <c r="A157" s="43" t="s">
         <v>63</v>
       </c>
       <c r="B157" s="4" t="s">
@@ -8830,7 +8842,7 @@
       </c>
     </row>
     <row r="158" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A158" s="41" t="s">
+      <c r="A158" s="43" t="s">
         <v>63</v>
       </c>
       <c r="B158" s="4" t="s">
@@ -8856,7 +8868,7 @@
       </c>
     </row>
     <row r="159" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A159" s="41" t="s">
+      <c r="A159" s="43" t="s">
         <v>63</v>
       </c>
       <c r="B159" s="4" t="s">
@@ -8884,7 +8896,7 @@
       </c>
     </row>
     <row r="160" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A160" s="41" t="s">
+      <c r="A160" s="43" t="s">
         <v>63</v>
       </c>
       <c r="B160" s="4" t="s">
@@ -8912,7 +8924,7 @@
       </c>
     </row>
     <row r="161" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A161" s="41" t="s">
+      <c r="A161" s="43" t="s">
         <v>64</v>
       </c>
       <c r="B161" s="4" t="s">
@@ -8930,7 +8942,7 @@
       <c r="L161" s="6"/>
     </row>
     <row r="162" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A162" s="41" t="s">
+      <c r="A162" s="43" t="s">
         <v>64</v>
       </c>
       <c r="B162" s="4" t="s">
@@ -8948,7 +8960,7 @@
       <c r="L162" s="6"/>
     </row>
     <row r="163" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A163" s="41" t="s">
+      <c r="A163" s="43" t="s">
         <v>64</v>
       </c>
       <c r="B163" s="4" t="s">
@@ -8968,7 +8980,7 @@
       <c r="L163" s="6"/>
     </row>
     <row r="164" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A164" s="41" t="s">
+      <c r="A164" s="43" t="s">
         <v>65</v>
       </c>
       <c r="B164" s="4" t="s">
@@ -8996,7 +9008,7 @@
       </c>
     </row>
     <row r="165" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A165" s="41" t="s">
+      <c r="A165" s="43" t="s">
         <v>65</v>
       </c>
       <c r="B165" s="4" t="s">
@@ -9034,7 +9046,7 @@
       </c>
     </row>
     <row r="166" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A166" s="41" t="s">
+      <c r="A166" s="43" t="s">
         <v>65</v>
       </c>
       <c r="B166" s="4" t="s">
@@ -9072,7 +9084,7 @@
       </c>
     </row>
     <row r="167" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A167" s="41" t="s">
+      <c r="A167" s="43" t="s">
         <v>65</v>
       </c>
       <c r="B167" s="4" t="s">
@@ -9110,7 +9122,7 @@
       </c>
     </row>
     <row r="168" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A168" s="41" t="s">
+      <c r="A168" s="43" t="s">
         <v>66</v>
       </c>
       <c r="B168" s="4" t="s">
@@ -9128,7 +9140,7 @@
       <c r="L168" s="6"/>
     </row>
     <row r="169" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A169" s="41" t="s">
+      <c r="A169" s="43" t="s">
         <v>66</v>
       </c>
       <c r="B169" s="4" t="s">
@@ -9166,7 +9178,7 @@
       </c>
     </row>
     <row r="170" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A170" s="41" t="s">
+      <c r="A170" s="43" t="s">
         <v>66</v>
       </c>
       <c r="B170" s="4" t="s">
@@ -9204,7 +9216,7 @@
       </c>
     </row>
     <row r="171" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A171" s="41" t="s">
+      <c r="A171" s="43" t="s">
         <v>66</v>
       </c>
       <c r="B171" s="4" t="s">
@@ -9242,7 +9254,7 @@
       </c>
     </row>
     <row r="172" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A172" s="41" t="s">
+      <c r="A172" s="43" t="s">
         <v>66</v>
       </c>
       <c r="B172" s="4" t="s">
@@ -9280,7 +9292,7 @@
       </c>
     </row>
     <row r="173" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A173" s="41" t="s">
+      <c r="A173" s="43" t="s">
         <v>67</v>
       </c>
       <c r="B173" s="4" t="s">
@@ -9318,7 +9330,7 @@
       </c>
     </row>
     <row r="174" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A174" s="41" t="s">
+      <c r="A174" s="43" t="s">
         <v>67</v>
       </c>
       <c r="B174" s="4" t="s">
@@ -9336,7 +9348,7 @@
       <c r="L174" s="6"/>
     </row>
     <row r="175" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A175" s="41" t="s">
+      <c r="A175" s="43" t="s">
         <v>67</v>
       </c>
       <c r="B175" s="4" t="s">
@@ -9354,7 +9366,7 @@
       <c r="L175" s="6"/>
     </row>
     <row r="176" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A176" s="41" t="s">
+      <c r="A176" s="43" t="s">
         <v>68</v>
       </c>
       <c r="B176" s="4" t="s">
@@ -9392,7 +9404,7 @@
       </c>
     </row>
     <row r="177" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A177" s="41" t="s">
+      <c r="A177" s="43" t="s">
         <v>68</v>
       </c>
       <c r="B177" s="4" t="s">
@@ -9424,7 +9436,7 @@
       <c r="L177" s="6"/>
     </row>
     <row r="178" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A178" s="41" t="s">
+      <c r="A178" s="43" t="s">
         <v>68</v>
       </c>
       <c r="B178" s="4" t="s">
@@ -9462,7 +9474,7 @@
       </c>
     </row>
     <row r="179" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A179" s="41" t="s">
+      <c r="A179" s="43" t="s">
         <v>69</v>
       </c>
       <c r="B179" s="4" t="s">
@@ -9500,7 +9512,7 @@
       </c>
     </row>
     <row r="180" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A180" s="41" t="s">
+      <c r="A180" s="43" t="s">
         <v>69</v>
       </c>
       <c r="B180" s="4" t="s">
@@ -9526,7 +9538,7 @@
       <c r="L180" s="6"/>
     </row>
     <row r="181" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A181" s="41" t="s">
+      <c r="A181" s="43" t="s">
         <v>69</v>
       </c>
       <c r="B181" s="4" t="s">
@@ -9564,7 +9576,7 @@
       </c>
     </row>
     <row r="182" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A182" s="41" t="s">
+      <c r="A182" s="43" t="s">
         <v>70</v>
       </c>
       <c r="B182" s="4" t="s">
@@ -9582,7 +9594,7 @@
       <c r="L182" s="6"/>
     </row>
     <row r="183" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A183" s="41" t="s">
+      <c r="A183" s="43" t="s">
         <v>70</v>
       </c>
       <c r="B183" s="4" t="s">
@@ -9600,7 +9612,7 @@
       <c r="L183" s="6"/>
     </row>
     <row r="184" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A184" s="41" t="s">
+      <c r="A184" s="43" t="s">
         <v>70</v>
       </c>
       <c r="B184" s="4" t="s">
@@ -9618,7 +9630,7 @@
       <c r="L184" s="6"/>
     </row>
     <row r="185" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A185" s="41" t="s">
+      <c r="A185" s="43" t="s">
         <v>70</v>
       </c>
       <c r="B185" s="4" t="s">
@@ -9636,7 +9648,7 @@
       <c r="L185" s="6"/>
     </row>
     <row r="186" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A186" s="41" t="s">
+      <c r="A186" s="43" t="s">
         <v>70</v>
       </c>
       <c r="B186" s="4" t="s">
@@ -9654,7 +9666,7 @@
       <c r="L186" s="6"/>
     </row>
     <row r="187" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A187" s="41" t="s">
+      <c r="A187" s="43" t="s">
         <v>71</v>
       </c>
       <c r="B187" s="4" t="s">
@@ -9672,7 +9684,7 @@
       <c r="L187" s="6"/>
     </row>
     <row r="188" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A188" s="41" t="s">
+      <c r="A188" s="43" t="s">
         <v>71</v>
       </c>
       <c r="B188" s="4" t="s">
@@ -9710,7 +9722,7 @@
       </c>
     </row>
     <row r="189" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A189" s="41" t="s">
+      <c r="A189" s="43" t="s">
         <v>71</v>
       </c>
       <c r="B189" s="4" t="s">
@@ -9748,7 +9760,7 @@
       </c>
     </row>
     <row r="190" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A190" s="41" t="s">
+      <c r="A190" s="43" t="s">
         <v>71</v>
       </c>
       <c r="B190" s="4" t="s">
@@ -9774,7 +9786,7 @@
       <c r="L190" s="6"/>
     </row>
     <row r="191" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A191" s="41" t="s">
+      <c r="A191" s="43" t="s">
         <v>71</v>
       </c>
       <c r="B191" s="4" t="s">
@@ -9812,7 +9824,7 @@
       </c>
     </row>
     <row r="192" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A192" s="41" t="s">
+      <c r="A192" s="43" t="s">
         <v>72</v>
       </c>
       <c r="B192" s="4" t="s">
@@ -9830,7 +9842,7 @@
       <c r="L192" s="6"/>
     </row>
     <row r="193" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A193" s="41" t="s">
+      <c r="A193" s="43" t="s">
         <v>72</v>
       </c>
       <c r="B193" s="4" t="s">
@@ -9868,7 +9880,7 @@
       </c>
     </row>
     <row r="194" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A194" s="41" t="s">
+      <c r="A194" s="43" t="s">
         <v>72</v>
       </c>
       <c r="B194" s="4" t="s">
@@ -9898,7 +9910,7 @@
       <c r="L194" s="6"/>
     </row>
     <row r="195" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A195" s="41" t="s">
+      <c r="A195" s="43" t="s">
         <v>72</v>
       </c>
       <c r="B195" s="4" t="s">
@@ -9936,7 +9948,7 @@
       </c>
     </row>
     <row r="196" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A196" s="41" t="s">
+      <c r="A196" s="43" t="s">
         <v>73</v>
       </c>
       <c r="B196" s="4" t="s">
@@ -9974,7 +9986,7 @@
       </c>
     </row>
     <row r="197" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A197" s="41" t="s">
+      <c r="A197" s="43" t="s">
         <v>73</v>
       </c>
       <c r="B197" s="4" t="s">
@@ -9992,7 +10004,7 @@
       <c r="L197" s="6"/>
     </row>
     <row r="198" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A198" s="41" t="s">
+      <c r="A198" s="43" t="s">
         <v>73</v>
       </c>
       <c r="B198" s="4" t="s">
@@ -10030,7 +10042,7 @@
       </c>
     </row>
     <row r="199" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A199" s="41" t="s">
+      <c r="A199" s="43" t="s">
         <v>74</v>
       </c>
       <c r="B199" s="4" t="s">
@@ -10068,7 +10080,7 @@
       </c>
     </row>
     <row r="200" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A200" s="41" t="s">
+      <c r="A200" s="43" t="s">
         <v>74</v>
       </c>
       <c r="B200" s="4" t="s">
@@ -10106,7 +10118,7 @@
       </c>
     </row>
     <row r="201" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A201" s="41" t="s">
+      <c r="A201" s="43" t="s">
         <v>74</v>
       </c>
       <c r="B201" s="4" t="s">
@@ -10144,7 +10156,7 @@
       </c>
     </row>
     <row r="202" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A202" s="41" t="s">
+      <c r="A202" s="43" t="s">
         <v>74</v>
       </c>
       <c r="B202" s="4" t="s">
@@ -10182,7 +10194,7 @@
       </c>
     </row>
     <row r="203" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A203" s="41" t="s">
+      <c r="A203" s="43" t="s">
         <v>74</v>
       </c>
       <c r="B203" s="4" t="s">
@@ -14278,12 +14290,40 @@
     </filterColumn>
   </autoFilter>
   <mergeCells count="52">
-    <mergeCell ref="A28:A30"/>
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="A7:A10"/>
-    <mergeCell ref="A11:A14"/>
-    <mergeCell ref="A17:A21"/>
-    <mergeCell ref="A22:A26"/>
+    <mergeCell ref="A187:A191"/>
+    <mergeCell ref="A192:A195"/>
+    <mergeCell ref="A196:A198"/>
+    <mergeCell ref="A199:A203"/>
+    <mergeCell ref="A164:A167"/>
+    <mergeCell ref="A168:A172"/>
+    <mergeCell ref="A173:A175"/>
+    <mergeCell ref="A176:A178"/>
+    <mergeCell ref="A179:A181"/>
+    <mergeCell ref="A182:A186"/>
+    <mergeCell ref="A161:A163"/>
+    <mergeCell ref="A120:A122"/>
+    <mergeCell ref="A123:A125"/>
+    <mergeCell ref="A126:A129"/>
+    <mergeCell ref="A130:A134"/>
+    <mergeCell ref="A135:A136"/>
+    <mergeCell ref="A137:A140"/>
+    <mergeCell ref="A142:A145"/>
+    <mergeCell ref="A146:A149"/>
+    <mergeCell ref="A150:A152"/>
+    <mergeCell ref="A153:A156"/>
+    <mergeCell ref="A157:A160"/>
+    <mergeCell ref="A114:A118"/>
+    <mergeCell ref="A75:A76"/>
+    <mergeCell ref="A78:A81"/>
+    <mergeCell ref="A82:A85"/>
+    <mergeCell ref="A86:A89"/>
+    <mergeCell ref="A90:A94"/>
+    <mergeCell ref="A95:A97"/>
+    <mergeCell ref="A98:A100"/>
+    <mergeCell ref="A101:A103"/>
+    <mergeCell ref="A104:A106"/>
+    <mergeCell ref="A107:A109"/>
+    <mergeCell ref="A110:A113"/>
     <mergeCell ref="A70:A74"/>
     <mergeCell ref="A31:A33"/>
     <mergeCell ref="A34:A36"/>
@@ -14296,40 +14336,12 @@
     <mergeCell ref="A58:A61"/>
     <mergeCell ref="A62:A64"/>
     <mergeCell ref="A65:A69"/>
-    <mergeCell ref="A114:A118"/>
-    <mergeCell ref="A75:A76"/>
-    <mergeCell ref="A78:A81"/>
-    <mergeCell ref="A82:A85"/>
-    <mergeCell ref="A86:A89"/>
-    <mergeCell ref="A90:A94"/>
-    <mergeCell ref="A95:A97"/>
-    <mergeCell ref="A98:A100"/>
-    <mergeCell ref="A101:A103"/>
-    <mergeCell ref="A104:A106"/>
-    <mergeCell ref="A107:A109"/>
-    <mergeCell ref="A110:A113"/>
-    <mergeCell ref="A161:A163"/>
-    <mergeCell ref="A120:A122"/>
-    <mergeCell ref="A123:A125"/>
-    <mergeCell ref="A126:A129"/>
-    <mergeCell ref="A130:A134"/>
-    <mergeCell ref="A135:A136"/>
-    <mergeCell ref="A137:A140"/>
-    <mergeCell ref="A142:A145"/>
-    <mergeCell ref="A146:A149"/>
-    <mergeCell ref="A150:A152"/>
-    <mergeCell ref="A153:A156"/>
-    <mergeCell ref="A157:A160"/>
-    <mergeCell ref="A187:A191"/>
-    <mergeCell ref="A192:A195"/>
-    <mergeCell ref="A196:A198"/>
-    <mergeCell ref="A199:A203"/>
-    <mergeCell ref="A164:A167"/>
-    <mergeCell ref="A168:A172"/>
-    <mergeCell ref="A173:A175"/>
-    <mergeCell ref="A176:A178"/>
-    <mergeCell ref="A179:A181"/>
-    <mergeCell ref="A182:A186"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="A7:A10"/>
+    <mergeCell ref="A11:A14"/>
+    <mergeCell ref="A17:A21"/>
+    <mergeCell ref="A22:A26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -18568,7 +18580,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="11" width="12.5703125" bestFit="1" customWidth="1"/>
@@ -18646,34 +18658,34 @@
         <v>140</v>
       </c>
       <c r="B3" s="37">
-        <v>24300000</v>
+        <v>243000000</v>
       </c>
       <c r="C3" s="37">
-        <v>26300000</v>
+        <v>263000000</v>
       </c>
       <c r="D3" s="37">
-        <v>26500000</v>
+        <v>265000000</v>
       </c>
       <c r="E3" s="37">
-        <v>25000000</v>
+        <v>250000000</v>
       </c>
       <c r="F3" s="37">
-        <v>24900000</v>
+        <v>249000000</v>
       </c>
       <c r="G3" s="37">
-        <v>24700000</v>
+        <v>247000000</v>
       </c>
       <c r="H3" s="37">
-        <v>25000000</v>
+        <v>250000000</v>
       </c>
       <c r="I3" s="37">
-        <v>24800000</v>
+        <v>248000000</v>
       </c>
       <c r="J3" s="37">
-        <v>25100000</v>
+        <v>251000000</v>
       </c>
       <c r="K3" s="37">
-        <v>25400000</v>
+        <v>254000000</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -18856,34 +18868,34 @@
         <v>116</v>
       </c>
       <c r="B9" s="37">
-        <v>173300000</v>
+        <v>1733000000</v>
       </c>
       <c r="C9" s="37">
-        <v>192100000</v>
+        <v>1921000000</v>
       </c>
       <c r="D9" s="37">
-        <v>207900000</v>
+        <v>2079000000</v>
       </c>
       <c r="E9" s="37">
-        <v>239100000</v>
+        <v>2391000000</v>
       </c>
       <c r="F9" s="37">
-        <v>260300000</v>
+        <v>2603000000</v>
       </c>
       <c r="G9" s="37">
-        <v>237100000</v>
+        <v>2371000000</v>
       </c>
       <c r="H9" s="37">
-        <v>225100000</v>
+        <v>2251000000</v>
       </c>
       <c r="I9" s="37">
-        <v>219800000</v>
+        <v>2198000000</v>
       </c>
       <c r="J9" s="37">
-        <v>215500000</v>
+        <v>2155000000</v>
       </c>
       <c r="K9" s="37">
-        <v>217800000</v>
+        <v>2178000000</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -18926,43 +18938,33 @@
         <v>147</v>
       </c>
       <c r="B11" s="25">
-        <f>B20*17</f>
         <v>1030200000</v>
       </c>
       <c r="C11" s="25">
-        <f t="shared" ref="C11:K11" si="0">C20*17</f>
         <v>1268200000</v>
       </c>
       <c r="D11" s="25">
-        <f t="shared" si="0"/>
         <v>1411000000</v>
       </c>
       <c r="E11" s="25">
-        <f t="shared" si="0"/>
         <v>1382100000</v>
       </c>
       <c r="F11" s="25">
-        <f t="shared" si="0"/>
         <v>1378700000</v>
       </c>
       <c r="G11" s="25">
-        <f t="shared" si="0"/>
         <v>1356600000</v>
       </c>
       <c r="H11" s="25">
-        <f t="shared" si="0"/>
         <v>1378700000</v>
       </c>
       <c r="I11" s="25">
-        <f t="shared" si="0"/>
         <v>1358300000</v>
       </c>
       <c r="J11" s="25">
-        <f t="shared" si="0"/>
         <v>1380400000</v>
       </c>
       <c r="K11" s="25">
-        <f t="shared" si="0"/>
         <v>1399100000</v>
       </c>
     </row>
@@ -19076,34 +19078,34 @@
         <v>151</v>
       </c>
       <c r="B15" s="37">
-        <v>104600000</v>
+        <v>1046000000</v>
       </c>
       <c r="C15" s="37">
-        <v>122100000</v>
+        <v>1221000000</v>
       </c>
       <c r="D15" s="37">
-        <v>131700000</v>
+        <v>1317000000</v>
       </c>
       <c r="E15" s="37">
-        <v>128600000</v>
+        <v>1286000000</v>
       </c>
       <c r="F15" s="37">
-        <v>128700000</v>
+        <v>1287000000</v>
       </c>
       <c r="G15" s="37">
-        <v>125200000</v>
+        <v>1252000000</v>
       </c>
       <c r="H15" s="37">
-        <v>127600000</v>
+        <v>1276000000</v>
       </c>
       <c r="I15" s="37">
-        <v>126000000</v>
+        <v>1260000000</v>
       </c>
       <c r="J15" s="37">
-        <v>127400000</v>
+        <v>1274000000</v>
       </c>
       <c r="K15" s="37">
-        <v>128200000</v>
+        <v>1282000000</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -19146,34 +19148,34 @@
         <v>153</v>
       </c>
       <c r="B17" s="25">
-        <v>500000</v>
+        <v>50000000</v>
       </c>
       <c r="C17" s="25">
-        <v>500000</v>
+        <v>50000000</v>
       </c>
       <c r="D17" s="25">
-        <v>700000</v>
+        <v>70000000</v>
       </c>
       <c r="E17" s="25">
-        <v>2000000</v>
+        <v>200000000</v>
       </c>
       <c r="F17" s="25">
-        <v>2500000</v>
+        <v>250000000</v>
       </c>
       <c r="G17" s="25">
-        <v>1800000</v>
+        <v>180000000</v>
       </c>
       <c r="H17" s="25">
-        <v>1200000</v>
+        <v>120000000</v>
       </c>
       <c r="I17" s="25">
-        <v>1200000</v>
+        <v>120000000</v>
       </c>
       <c r="J17" s="25">
-        <v>900000</v>
+        <v>90000000</v>
       </c>
       <c r="K17" s="25">
-        <v>1000000</v>
+        <v>100000000</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -19181,34 +19183,34 @@
         <v>156</v>
       </c>
       <c r="B18" s="37">
-        <v>5800000</v>
+        <v>58000000</v>
       </c>
       <c r="C18" s="37">
-        <v>6700000</v>
+        <v>67000000</v>
       </c>
       <c r="D18" s="37">
-        <v>7500000</v>
+        <v>75000000</v>
       </c>
       <c r="E18" s="37">
-        <v>7400000</v>
+        <v>74000000</v>
       </c>
       <c r="F18" s="37">
-        <v>7900000</v>
+        <v>79000000</v>
       </c>
       <c r="G18" s="37">
-        <v>7900000</v>
+        <v>79000000</v>
       </c>
       <c r="H18" s="37">
-        <v>8000000</v>
+        <v>80000000</v>
       </c>
       <c r="I18" s="37">
-        <v>7800000</v>
+        <v>78000000</v>
       </c>
       <c r="J18" s="37">
-        <v>7800000</v>
+        <v>78000000</v>
       </c>
       <c r="K18" s="37">
-        <v>7900000</v>
+        <v>79000000</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
@@ -19224,63 +19226,43 @@
       <c r="K19" s="25"/>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B20" s="37">
-        <v>60600000</v>
-      </c>
-      <c r="C20" s="37">
-        <v>74600000</v>
-      </c>
-      <c r="D20" s="37">
-        <v>83000000</v>
-      </c>
-      <c r="E20" s="37">
-        <v>81300000</v>
-      </c>
-      <c r="F20" s="37">
-        <v>81100000</v>
-      </c>
-      <c r="G20" s="37">
-        <v>79800000</v>
-      </c>
-      <c r="H20" s="37">
-        <v>81100000</v>
-      </c>
-      <c r="I20" s="37">
-        <v>79900000</v>
-      </c>
-      <c r="J20" s="37">
-        <v>81200000</v>
-      </c>
-      <c r="K20" s="37">
-        <v>82300000</v>
-      </c>
+      <c r="B20" s="37"/>
+      <c r="C20" s="37"/>
+      <c r="D20" s="37"/>
+      <c r="E20" s="37"/>
+      <c r="F20" s="37"/>
+      <c r="G20" s="37"/>
+      <c r="H20" s="37"/>
+      <c r="I20" s="37"/>
+      <c r="J20" s="37"/>
+      <c r="K20" s="37"/>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="25"/>
-      <c r="J21" s="25"/>
-      <c r="K21" s="25"/>
+      <c r="B21" s="42"/>
+      <c r="C21" s="42"/>
+      <c r="D21" s="42"/>
+      <c r="E21" s="42"/>
+      <c r="F21" s="42"/>
+      <c r="G21" s="42"/>
+      <c r="H21" s="42"/>
+      <c r="I21" s="42"/>
+      <c r="J21" s="42"/>
+      <c r="K21" s="42"/>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="25"/>
-      <c r="J22" s="25"/>
-      <c r="K22" s="25"/>
+      <c r="B22" s="41"/>
+      <c r="C22" s="42"/>
+      <c r="D22" s="42"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="42"/>
+      <c r="G22" s="42"/>
+      <c r="H22" s="42"/>
+      <c r="I22" s="42"/>
+      <c r="J22" s="42"/>
+      <c r="K22" s="42"/>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="25"/>
+      <c r="B23" s="37"/>
       <c r="C23" s="25"/>
       <c r="D23" s="25"/>
       <c r="E23" s="40"/>

</xml_diff>

<commit_message>
added tender start and end horizon
</commit_message>
<xml_diff>
--- a/production_capacity_updated.xlsx
+++ b/production_capacity_updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="137" documentId="13_ncr:1_{68782C53-48E3-42CA-912A-5E0671CC39DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{49F25625-B636-41FB-B8B0-30066A052327}"/>
+  <xr:revisionPtr revIDLastSave="155" documentId="13_ncr:1_{68782C53-48E3-42CA-912A-5E0671CC39DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E313997-B984-44EE-A796-E33C8848E5C0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="4" xr2:uid="{752E71BE-3FD4-4CCA-ABF0-6C5710D300B4}"/>
   </bookViews>
@@ -957,7 +957,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -1045,6 +1045,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -19467,7 +19470,9 @@
       <c r="K20" s="43"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B21" s="43"/>
+      <c r="B21" s="43">
+        <v>43365104</v>
+      </c>
       <c r="C21" s="42"/>
       <c r="D21" s="42"/>
       <c r="E21" s="25"/>
@@ -19479,7 +19484,9 @@
       <c r="K21" s="25"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B22" s="42"/>
+      <c r="B22" s="48">
+        <v>61220888</v>
+      </c>
       <c r="C22" s="42"/>
       <c r="D22" s="42"/>
       <c r="E22" s="25"/>
@@ -19491,7 +19498,10 @@
       <c r="K22" s="25"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B23" s="25"/>
+      <c r="B23" s="25">
+        <f>B22+B21</f>
+        <v>104585992</v>
+      </c>
       <c r="C23" s="25"/>
       <c r="D23" s="25"/>
       <c r="E23" s="40"/>
@@ -19503,7 +19513,10 @@
       <c r="K23" s="25"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="25"/>
+      <c r="B24" s="25">
+        <f>B16-B23</f>
+        <v>14008</v>
+      </c>
       <c r="C24" s="25"/>
       <c r="D24" s="25"/>
       <c r="E24" s="25"/>

</xml_diff>